<commit_message>
making access codes private
</commit_message>
<xml_diff>
--- a/finance_data.xlsx
+++ b/finance_data.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Balances" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key &amp; Instructions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access Codes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +122,44 @@
       <color rgb="00444444"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007B0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -149,8 +186,48 @@
         <fgColor rgb="00FFF8DC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4B5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9F9F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -172,11 +249,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -298,6 +419,69 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -683,6 +867,14 @@
           <t>ROSTER &amp; ACCESS CODES — Ultimate Frisbee Team</t>
         </is>
       </c>
+      <c r="B1" s="53" t="n"/>
+      <c r="C1" s="53" t="n"/>
+      <c r="D1" s="53" t="n"/>
+      <c r="E1" s="53" t="n"/>
+      <c r="F1" s="53" t="n"/>
+      <c r="G1" s="53" t="n"/>
+      <c r="H1" s="53" t="n"/>
+      <c r="I1" s="54" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
@@ -761,9 +953,9 @@
           <t>Full Name</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Access Code</t>
+      <c r="B6" s="55" t="inlineStr">
+        <is>
+          <t>Code (→ see 'Access Codes' tab)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -808,7 +1000,7 @@
           <t>Alex Johnson</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="56" t="inlineStr">
         <is>
           <t>AJ2024</t>
         </is>
@@ -845,7 +1037,7 @@
           <t>Sam Rivera</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="56" t="inlineStr">
         <is>
           <t>SR2024</t>
         </is>
@@ -882,7 +1074,7 @@
           <t>Jordan Lee</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="56" t="inlineStr">
         <is>
           <t>JL2024</t>
         </is>
@@ -923,7 +1115,7 @@
           <t>Coach Kim</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="56" t="inlineStr">
         <is>
           <t>CK2024</t>
         </is>
@@ -956,7 +1148,7 @@
           <t>Taylor Smith</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="56" t="inlineStr">
         <is>
           <t>TS2024</t>
         </is>
@@ -989,7 +1181,7 @@
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="10" t="n"/>
-      <c r="B12" s="11" t="n"/>
+      <c r="B12" s="57" t="n"/>
       <c r="C12" s="10" t="n"/>
       <c r="D12" s="12" t="n"/>
       <c r="E12" s="13" t="n"/>
@@ -1000,7 +1192,7 @@
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="14" t="n"/>
-      <c r="B13" s="15" t="n"/>
+      <c r="B13" s="57" t="n"/>
       <c r="C13" s="14" t="n"/>
       <c r="D13" s="16" t="n"/>
       <c r="E13" s="17" t="n"/>
@@ -1011,7 +1203,7 @@
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="10" t="n"/>
-      <c r="B14" s="11" t="n"/>
+      <c r="B14" s="57" t="n"/>
       <c r="C14" s="10" t="n"/>
       <c r="D14" s="12" t="n"/>
       <c r="E14" s="13" t="n"/>
@@ -1022,7 +1214,7 @@
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="14" t="n"/>
-      <c r="B15" s="15" t="n"/>
+      <c r="B15" s="57" t="n"/>
       <c r="C15" s="14" t="n"/>
       <c r="D15" s="16" t="n"/>
       <c r="E15" s="17" t="n"/>
@@ -1033,7 +1225,7 @@
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="10" t="n"/>
-      <c r="B16" s="11" t="n"/>
+      <c r="B16" s="57" t="n"/>
       <c r="C16" s="10" t="n"/>
       <c r="D16" s="12" t="n"/>
       <c r="E16" s="13" t="n"/>
@@ -1044,7 +1236,7 @@
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="14" t="n"/>
-      <c r="B17" s="15" t="n"/>
+      <c r="B17" s="57" t="n"/>
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="16" t="n"/>
       <c r="E17" s="17" t="n"/>
@@ -1055,7 +1247,7 @@
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="10" t="n"/>
-      <c r="B18" s="11" t="n"/>
+      <c r="B18" s="57" t="n"/>
       <c r="C18" s="10" t="n"/>
       <c r="D18" s="12" t="n"/>
       <c r="E18" s="13" t="n"/>
@@ -1066,7 +1258,7 @@
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="14" t="n"/>
-      <c r="B19" s="15" t="n"/>
+      <c r="B19" s="57" t="n"/>
       <c r="C19" s="14" t="n"/>
       <c r="D19" s="16" t="n"/>
       <c r="E19" s="17" t="n"/>
@@ -1077,7 +1269,7 @@
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="10" t="n"/>
-      <c r="B20" s="11" t="n"/>
+      <c r="B20" s="57" t="n"/>
       <c r="C20" s="10" t="n"/>
       <c r="D20" s="12" t="n"/>
       <c r="E20" s="13" t="n"/>
@@ -1088,7 +1280,7 @@
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="14" t="n"/>
-      <c r="B21" s="15" t="n"/>
+      <c r="B21" s="57" t="n"/>
       <c r="C21" s="14" t="n"/>
       <c r="D21" s="16" t="n"/>
       <c r="E21" s="17" t="n"/>
@@ -1099,7 +1291,7 @@
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="10" t="n"/>
-      <c r="B22" s="11" t="n"/>
+      <c r="B22" s="57" t="n"/>
       <c r="C22" s="10" t="n"/>
       <c r="D22" s="12" t="n"/>
       <c r="E22" s="13" t="n"/>
@@ -1110,7 +1302,7 @@
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="14" t="n"/>
-      <c r="B23" s="15" t="n"/>
+      <c r="B23" s="57" t="n"/>
       <c r="C23" s="14" t="n"/>
       <c r="D23" s="16" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -1121,7 +1313,7 @@
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="10" t="n"/>
-      <c r="B24" s="11" t="n"/>
+      <c r="B24" s="57" t="n"/>
       <c r="C24" s="10" t="n"/>
       <c r="D24" s="12" t="n"/>
       <c r="E24" s="13" t="n"/>
@@ -1132,7 +1324,7 @@
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="14" t="n"/>
-      <c r="B25" s="15" t="n"/>
+      <c r="B25" s="57" t="n"/>
       <c r="C25" s="14" t="n"/>
       <c r="D25" s="16" t="n"/>
       <c r="E25" s="17" t="n"/>
@@ -1143,7 +1335,7 @@
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="10" t="n"/>
-      <c r="B26" s="11" t="n"/>
+      <c r="B26" s="57" t="n"/>
       <c r="C26" s="10" t="n"/>
       <c r="D26" s="12" t="n"/>
       <c r="E26" s="13" t="n"/>
@@ -1154,7 +1346,7 @@
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="14" t="n"/>
-      <c r="B27" s="15" t="n"/>
+      <c r="B27" s="57" t="n"/>
       <c r="C27" s="14" t="n"/>
       <c r="D27" s="16" t="n"/>
       <c r="E27" s="17" t="n"/>
@@ -1165,7 +1357,7 @@
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="10" t="n"/>
-      <c r="B28" s="11" t="n"/>
+      <c r="B28" s="57" t="n"/>
       <c r="C28" s="10" t="n"/>
       <c r="D28" s="12" t="n"/>
       <c r="E28" s="13" t="n"/>
@@ -1176,7 +1368,7 @@
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="14" t="n"/>
-      <c r="B29" s="15" t="n"/>
+      <c r="B29" s="57" t="n"/>
       <c r="C29" s="14" t="n"/>
       <c r="D29" s="16" t="n"/>
       <c r="E29" s="17" t="n"/>
@@ -1187,7 +1379,7 @@
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="10" t="n"/>
-      <c r="B30" s="11" t="n"/>
+      <c r="B30" s="57" t="n"/>
       <c r="C30" s="10" t="n"/>
       <c r="D30" s="12" t="n"/>
       <c r="E30" s="13" t="n"/>
@@ -1198,7 +1390,7 @@
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="14" t="n"/>
-      <c r="B31" s="15" t="n"/>
+      <c r="B31" s="57" t="n"/>
       <c r="C31" s="14" t="n"/>
       <c r="D31" s="16" t="n"/>
       <c r="E31" s="17" t="n"/>
@@ -1209,7 +1401,7 @@
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="10" t="n"/>
-      <c r="B32" s="11" t="n"/>
+      <c r="B32" s="57" t="n"/>
       <c r="C32" s="10" t="n"/>
       <c r="D32" s="12" t="n"/>
       <c r="E32" s="13" t="n"/>
@@ -1220,7 +1412,7 @@
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="14" t="n"/>
-      <c r="B33" s="15" t="n"/>
+      <c r="B33" s="57" t="n"/>
       <c r="C33" s="14" t="n"/>
       <c r="D33" s="16" t="n"/>
       <c r="E33" s="17" t="n"/>
@@ -1231,7 +1423,7 @@
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="10" t="n"/>
-      <c r="B34" s="11" t="n"/>
+      <c r="B34" s="57" t="n"/>
       <c r="C34" s="10" t="n"/>
       <c r="D34" s="12" t="n"/>
       <c r="E34" s="13" t="n"/>
@@ -1242,7 +1434,7 @@
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="14" t="n"/>
-      <c r="B35" s="15" t="n"/>
+      <c r="B35" s="57" t="n"/>
       <c r="C35" s="14" t="n"/>
       <c r="D35" s="16" t="n"/>
       <c r="E35" s="17" t="n"/>
@@ -1253,7 +1445,7 @@
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="10" t="n"/>
-      <c r="B36" s="11" t="n"/>
+      <c r="B36" s="57" t="n"/>
       <c r="C36" s="10" t="n"/>
       <c r="D36" s="12" t="n"/>
       <c r="E36" s="13" t="n"/>
@@ -1264,7 +1456,7 @@
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="14" t="n"/>
-      <c r="B37" s="15" t="n"/>
+      <c r="B37" s="57" t="n"/>
       <c r="C37" s="14" t="n"/>
       <c r="D37" s="16" t="n"/>
       <c r="E37" s="17" t="n"/>
@@ -1275,7 +1467,7 @@
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="10" t="n"/>
-      <c r="B38" s="11" t="n"/>
+      <c r="B38" s="57" t="n"/>
       <c r="C38" s="10" t="n"/>
       <c r="D38" s="12" t="n"/>
       <c r="E38" s="13" t="n"/>
@@ -1286,7 +1478,7 @@
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="14" t="n"/>
-      <c r="B39" s="15" t="n"/>
+      <c r="B39" s="57" t="n"/>
       <c r="C39" s="14" t="n"/>
       <c r="D39" s="16" t="n"/>
       <c r="E39" s="17" t="n"/>
@@ -1297,7 +1489,7 @@
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="10" t="n"/>
-      <c r="B40" s="11" t="n"/>
+      <c r="B40" s="57" t="n"/>
       <c r="C40" s="10" t="n"/>
       <c r="D40" s="12" t="n"/>
       <c r="E40" s="13" t="n"/>
@@ -1308,7 +1500,7 @@
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="14" t="n"/>
-      <c r="B41" s="15" t="n"/>
+      <c r="B41" s="57" t="n"/>
       <c r="C41" s="14" t="n"/>
       <c r="D41" s="16" t="n"/>
       <c r="E41" s="17" t="n"/>
@@ -1319,7 +1511,7 @@
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="10" t="n"/>
-      <c r="B42" s="11" t="n"/>
+      <c r="B42" s="57" t="n"/>
       <c r="C42" s="10" t="n"/>
       <c r="D42" s="12" t="n"/>
       <c r="E42" s="13" t="n"/>
@@ -1330,7 +1522,7 @@
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="14" t="n"/>
-      <c r="B43" s="15" t="n"/>
+      <c r="B43" s="57" t="n"/>
       <c r="C43" s="14" t="n"/>
       <c r="D43" s="16" t="n"/>
       <c r="E43" s="17" t="n"/>
@@ -1341,7 +1533,7 @@
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="10" t="n"/>
-      <c r="B44" s="11" t="n"/>
+      <c r="B44" s="57" t="n"/>
       <c r="C44" s="10" t="n"/>
       <c r="D44" s="12" t="n"/>
       <c r="E44" s="13" t="n"/>
@@ -1352,7 +1544,7 @@
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="14" t="n"/>
-      <c r="B45" s="15" t="n"/>
+      <c r="B45" s="57" t="n"/>
       <c r="C45" s="14" t="n"/>
       <c r="D45" s="16" t="n"/>
       <c r="E45" s="17" t="n"/>
@@ -1363,7 +1555,7 @@
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="10" t="n"/>
-      <c r="B46" s="11" t="n"/>
+      <c r="B46" s="57" t="n"/>
       <c r="C46" s="10" t="n"/>
       <c r="D46" s="12" t="n"/>
       <c r="E46" s="13" t="n"/>
@@ -1374,7 +1566,7 @@
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="14" t="n"/>
-      <c r="B47" s="15" t="n"/>
+      <c r="B47" s="57" t="n"/>
       <c r="C47" s="14" t="n"/>
       <c r="D47" s="16" t="n"/>
       <c r="E47" s="17" t="n"/>
@@ -1385,7 +1577,7 @@
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="10" t="n"/>
-      <c r="B48" s="11" t="n"/>
+      <c r="B48" s="57" t="n"/>
       <c r="C48" s="10" t="n"/>
       <c r="D48" s="12" t="n"/>
       <c r="E48" s="13" t="n"/>
@@ -1396,7 +1588,7 @@
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="14" t="n"/>
-      <c r="B49" s="15" t="n"/>
+      <c r="B49" s="57" t="n"/>
       <c r="C49" s="14" t="n"/>
       <c r="D49" s="16" t="n"/>
       <c r="E49" s="17" t="n"/>
@@ -1407,7 +1599,7 @@
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="10" t="n"/>
-      <c r="B50" s="11" t="n"/>
+      <c r="B50" s="57" t="n"/>
       <c r="C50" s="10" t="n"/>
       <c r="D50" s="12" t="n"/>
       <c r="E50" s="13" t="n"/>
@@ -1418,7 +1610,7 @@
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="14" t="n"/>
-      <c r="B51" s="15" t="n"/>
+      <c r="B51" s="57" t="n"/>
       <c r="C51" s="14" t="n"/>
       <c r="D51" s="16" t="n"/>
       <c r="E51" s="17" t="n"/>
@@ -1429,7 +1621,7 @@
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="10" t="n"/>
-      <c r="B52" s="11" t="n"/>
+      <c r="B52" s="57" t="n"/>
       <c r="C52" s="10" t="n"/>
       <c r="D52" s="12" t="n"/>
       <c r="E52" s="13" t="n"/>
@@ -1440,7 +1632,7 @@
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="14" t="n"/>
-      <c r="B53" s="15" t="n"/>
+      <c r="B53" s="57" t="n"/>
       <c r="C53" s="14" t="n"/>
       <c r="D53" s="16" t="n"/>
       <c r="E53" s="17" t="n"/>
@@ -1451,7 +1643,7 @@
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="10" t="n"/>
-      <c r="B54" s="11" t="n"/>
+      <c r="B54" s="57" t="n"/>
       <c r="C54" s="10" t="n"/>
       <c r="D54" s="12" t="n"/>
       <c r="E54" s="13" t="n"/>
@@ -1462,7 +1654,7 @@
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="14" t="n"/>
-      <c r="B55" s="15" t="n"/>
+      <c r="B55" s="57" t="n"/>
       <c r="C55" s="14" t="n"/>
       <c r="D55" s="16" t="n"/>
       <c r="E55" s="17" t="n"/>
@@ -1473,7 +1665,7 @@
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="10" t="n"/>
-      <c r="B56" s="11" t="n"/>
+      <c r="B56" s="57" t="n"/>
       <c r="C56" s="10" t="n"/>
       <c r="D56" s="12" t="n"/>
       <c r="E56" s="13" t="n"/>
@@ -1484,7 +1676,7 @@
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="14" t="n"/>
-      <c r="B57" s="15" t="n"/>
+      <c r="B57" s="57" t="n"/>
       <c r="C57" s="14" t="n"/>
       <c r="D57" s="16" t="n"/>
       <c r="E57" s="17" t="n"/>
@@ -1495,7 +1687,7 @@
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="10" t="n"/>
-      <c r="B58" s="11" t="n"/>
+      <c r="B58" s="57" t="n"/>
       <c r="C58" s="10" t="n"/>
       <c r="D58" s="12" t="n"/>
       <c r="E58" s="13" t="n"/>
@@ -1506,7 +1698,7 @@
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="14" t="n"/>
-      <c r="B59" s="15" t="n"/>
+      <c r="B59" s="57" t="n"/>
       <c r="C59" s="14" t="n"/>
       <c r="D59" s="16" t="n"/>
       <c r="E59" s="17" t="n"/>
@@ -1517,7 +1709,7 @@
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="10" t="n"/>
-      <c r="B60" s="11" t="n"/>
+      <c r="B60" s="57" t="n"/>
       <c r="C60" s="10" t="n"/>
       <c r="D60" s="12" t="n"/>
       <c r="E60" s="13" t="n"/>
@@ -1528,7 +1720,7 @@
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="14" t="n"/>
-      <c r="B61" s="15" t="n"/>
+      <c r="B61" s="57" t="n"/>
       <c r="C61" s="14" t="n"/>
       <c r="D61" s="16" t="n"/>
       <c r="E61" s="17" t="n"/>
@@ -1539,7 +1731,7 @@
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="10" t="n"/>
-      <c r="B62" s="11" t="n"/>
+      <c r="B62" s="57" t="n"/>
       <c r="C62" s="10" t="n"/>
       <c r="D62" s="12" t="n"/>
       <c r="E62" s="13" t="n"/>
@@ -1550,7 +1742,7 @@
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="14" t="n"/>
-      <c r="B63" s="15" t="n"/>
+      <c r="B63" s="57" t="n"/>
       <c r="C63" s="14" t="n"/>
       <c r="D63" s="16" t="n"/>
       <c r="E63" s="17" t="n"/>
@@ -1561,7 +1753,7 @@
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="10" t="n"/>
-      <c r="B64" s="11" t="n"/>
+      <c r="B64" s="57" t="n"/>
       <c r="C64" s="10" t="n"/>
       <c r="D64" s="12" t="n"/>
       <c r="E64" s="13" t="n"/>
@@ -1572,7 +1764,7 @@
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="14" t="n"/>
-      <c r="B65" s="15" t="n"/>
+      <c r="B65" s="57" t="n"/>
       <c r="C65" s="14" t="n"/>
       <c r="D65" s="16" t="n"/>
       <c r="E65" s="17" t="n"/>
@@ -1583,7 +1775,7 @@
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="10" t="n"/>
-      <c r="B66" s="11" t="n"/>
+      <c r="B66" s="57" t="n"/>
       <c r="C66" s="10" t="n"/>
       <c r="D66" s="12" t="n"/>
       <c r="E66" s="13" t="n"/>
@@ -1594,7 +1786,7 @@
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="14" t="n"/>
-      <c r="B67" s="15" t="n"/>
+      <c r="B67" s="57" t="n"/>
       <c r="C67" s="14" t="n"/>
       <c r="D67" s="16" t="n"/>
       <c r="E67" s="17" t="n"/>
@@ -1605,7 +1797,7 @@
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="10" t="n"/>
-      <c r="B68" s="11" t="n"/>
+      <c r="B68" s="57" t="n"/>
       <c r="C68" s="10" t="n"/>
       <c r="D68" s="12" t="n"/>
       <c r="E68" s="13" t="n"/>
@@ -1616,7 +1808,7 @@
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="14" t="n"/>
-      <c r="B69" s="15" t="n"/>
+      <c r="B69" s="57" t="n"/>
       <c r="C69" s="14" t="n"/>
       <c r="D69" s="16" t="n"/>
       <c r="E69" s="17" t="n"/>
@@ -1627,7 +1819,7 @@
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="10" t="n"/>
-      <c r="B70" s="11" t="n"/>
+      <c r="B70" s="57" t="n"/>
       <c r="C70" s="10" t="n"/>
       <c r="D70" s="12" t="n"/>
       <c r="E70" s="13" t="n"/>
@@ -1638,7 +1830,7 @@
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="14" t="n"/>
-      <c r="B71" s="15" t="n"/>
+      <c r="B71" s="57" t="n"/>
       <c r="C71" s="14" t="n"/>
       <c r="D71" s="16" t="n"/>
       <c r="E71" s="17" t="n"/>
@@ -1649,7 +1841,7 @@
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="10" t="n"/>
-      <c r="B72" s="11" t="n"/>
+      <c r="B72" s="57" t="n"/>
       <c r="C72" s="10" t="n"/>
       <c r="D72" s="12" t="n"/>
       <c r="E72" s="13" t="n"/>
@@ -1660,7 +1852,7 @@
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="14" t="n"/>
-      <c r="B73" s="15" t="n"/>
+      <c r="B73" s="57" t="n"/>
       <c r="C73" s="14" t="n"/>
       <c r="D73" s="16" t="n"/>
       <c r="E73" s="17" t="n"/>
@@ -1671,7 +1863,7 @@
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="10" t="n"/>
-      <c r="B74" s="11" t="n"/>
+      <c r="B74" s="57" t="n"/>
       <c r="C74" s="10" t="n"/>
       <c r="D74" s="12" t="n"/>
       <c r="E74" s="13" t="n"/>
@@ -1682,7 +1874,7 @@
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="14" t="n"/>
-      <c r="B75" s="15" t="n"/>
+      <c r="B75" s="57" t="n"/>
       <c r="C75" s="14" t="n"/>
       <c r="D75" s="16" t="n"/>
       <c r="E75" s="17" t="n"/>
@@ -1693,7 +1885,7 @@
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="10" t="n"/>
-      <c r="B76" s="11" t="n"/>
+      <c r="B76" s="57" t="n"/>
       <c r="C76" s="10" t="n"/>
       <c r="D76" s="12" t="n"/>
       <c r="E76" s="13" t="n"/>
@@ -1704,7 +1896,7 @@
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="14" t="n"/>
-      <c r="B77" s="15" t="n"/>
+      <c r="B77" s="57" t="n"/>
       <c r="C77" s="14" t="n"/>
       <c r="D77" s="16" t="n"/>
       <c r="E77" s="17" t="n"/>
@@ -1715,7 +1907,7 @@
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="10" t="n"/>
-      <c r="B78" s="11" t="n"/>
+      <c r="B78" s="57" t="n"/>
       <c r="C78" s="10" t="n"/>
       <c r="D78" s="12" t="n"/>
       <c r="E78" s="13" t="n"/>
@@ -1726,7 +1918,7 @@
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="14" t="n"/>
-      <c r="B79" s="15" t="n"/>
+      <c r="B79" s="57" t="n"/>
       <c r="C79" s="14" t="n"/>
       <c r="D79" s="16" t="n"/>
       <c r="E79" s="17" t="n"/>
@@ -1737,7 +1929,7 @@
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="10" t="n"/>
-      <c r="B80" s="11" t="n"/>
+      <c r="B80" s="57" t="n"/>
       <c r="C80" s="10" t="n"/>
       <c r="D80" s="12" t="n"/>
       <c r="E80" s="13" t="n"/>
@@ -1748,7 +1940,7 @@
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="14" t="n"/>
-      <c r="B81" s="15" t="n"/>
+      <c r="B81" s="57" t="n"/>
       <c r="C81" s="14" t="n"/>
       <c r="D81" s="16" t="n"/>
       <c r="E81" s="17" t="n"/>
@@ -1759,7 +1951,7 @@
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="10" t="n"/>
-      <c r="B82" s="11" t="n"/>
+      <c r="B82" s="57" t="n"/>
       <c r="C82" s="10" t="n"/>
       <c r="D82" s="12" t="n"/>
       <c r="E82" s="13" t="n"/>
@@ -1770,7 +1962,7 @@
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="14" t="n"/>
-      <c r="B83" s="15" t="n"/>
+      <c r="B83" s="57" t="n"/>
       <c r="C83" s="14" t="n"/>
       <c r="D83" s="16" t="n"/>
       <c r="E83" s="17" t="n"/>
@@ -1781,7 +1973,7 @@
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="10" t="n"/>
-      <c r="B84" s="11" t="n"/>
+      <c r="B84" s="57" t="n"/>
       <c r="C84" s="10" t="n"/>
       <c r="D84" s="12" t="n"/>
       <c r="E84" s="13" t="n"/>
@@ -1792,7 +1984,7 @@
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="14" t="n"/>
-      <c r="B85" s="15" t="n"/>
+      <c r="B85" s="57" t="n"/>
       <c r="C85" s="14" t="n"/>
       <c r="D85" s="16" t="n"/>
       <c r="E85" s="17" t="n"/>
@@ -1803,7 +1995,7 @@
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="10" t="n"/>
-      <c r="B86" s="11" t="n"/>
+      <c r="B86" s="57" t="n"/>
       <c r="C86" s="10" t="n"/>
       <c r="D86" s="12" t="n"/>
       <c r="E86" s="13" t="n"/>
@@ -1814,7 +2006,7 @@
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="14" t="n"/>
-      <c r="B87" s="15" t="n"/>
+      <c r="B87" s="57" t="n"/>
       <c r="C87" s="14" t="n"/>
       <c r="D87" s="16" t="n"/>
       <c r="E87" s="17" t="n"/>
@@ -1825,7 +2017,7 @@
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="10" t="n"/>
-      <c r="B88" s="11" t="n"/>
+      <c r="B88" s="57" t="n"/>
       <c r="C88" s="10" t="n"/>
       <c r="D88" s="12" t="n"/>
       <c r="E88" s="13" t="n"/>
@@ -1836,7 +2028,7 @@
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="14" t="n"/>
-      <c r="B89" s="15" t="n"/>
+      <c r="B89" s="57" t="n"/>
       <c r="C89" s="14" t="n"/>
       <c r="D89" s="16" t="n"/>
       <c r="E89" s="17" t="n"/>
@@ -1847,7 +2039,7 @@
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="10" t="n"/>
-      <c r="B90" s="11" t="n"/>
+      <c r="B90" s="57" t="n"/>
       <c r="C90" s="10" t="n"/>
       <c r="D90" s="12" t="n"/>
       <c r="E90" s="13" t="n"/>
@@ -1858,7 +2050,7 @@
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="14" t="n"/>
-      <c r="B91" s="15" t="n"/>
+      <c r="B91" s="57" t="n"/>
       <c r="C91" s="14" t="n"/>
       <c r="D91" s="16" t="n"/>
       <c r="E91" s="17" t="n"/>
@@ -1869,7 +2061,7 @@
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="10" t="n"/>
-      <c r="B92" s="11" t="n"/>
+      <c r="B92" s="57" t="n"/>
       <c r="C92" s="10" t="n"/>
       <c r="D92" s="12" t="n"/>
       <c r="E92" s="13" t="n"/>
@@ -1880,7 +2072,7 @@
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="14" t="n"/>
-      <c r="B93" s="15" t="n"/>
+      <c r="B93" s="57" t="n"/>
       <c r="C93" s="14" t="n"/>
       <c r="D93" s="16" t="n"/>
       <c r="E93" s="17" t="n"/>
@@ -1891,7 +2083,7 @@
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="10" t="n"/>
-      <c r="B94" s="11" t="n"/>
+      <c r="B94" s="57" t="n"/>
       <c r="C94" s="10" t="n"/>
       <c r="D94" s="12" t="n"/>
       <c r="E94" s="13" t="n"/>
@@ -1902,7 +2094,7 @@
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="14" t="n"/>
-      <c r="B95" s="15" t="n"/>
+      <c r="B95" s="57" t="n"/>
       <c r="C95" s="14" t="n"/>
       <c r="D95" s="16" t="n"/>
       <c r="E95" s="17" t="n"/>
@@ -1913,7 +2105,7 @@
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="10" t="n"/>
-      <c r="B96" s="11" t="n"/>
+      <c r="B96" s="57" t="n"/>
       <c r="C96" s="10" t="n"/>
       <c r="D96" s="12" t="n"/>
       <c r="E96" s="13" t="n"/>
@@ -1924,7 +2116,7 @@
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="14" t="n"/>
-      <c r="B97" s="15" t="n"/>
+      <c r="B97" s="57" t="n"/>
       <c r="C97" s="14" t="n"/>
       <c r="D97" s="16" t="n"/>
       <c r="E97" s="17" t="n"/>
@@ -1935,7 +2127,7 @@
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="10" t="n"/>
-      <c r="B98" s="11" t="n"/>
+      <c r="B98" s="57" t="n"/>
       <c r="C98" s="10" t="n"/>
       <c r="D98" s="12" t="n"/>
       <c r="E98" s="13" t="n"/>
@@ -1946,7 +2138,7 @@
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="14" t="n"/>
-      <c r="B99" s="15" t="n"/>
+      <c r="B99" s="57" t="n"/>
       <c r="C99" s="14" t="n"/>
       <c r="D99" s="16" t="n"/>
       <c r="E99" s="17" t="n"/>
@@ -1957,7 +2149,7 @@
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="10" t="n"/>
-      <c r="B100" s="11" t="n"/>
+      <c r="B100" s="57" t="n"/>
       <c r="C100" s="10" t="n"/>
       <c r="D100" s="12" t="n"/>
       <c r="E100" s="13" t="n"/>
@@ -1968,7 +2160,7 @@
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="14" t="n"/>
-      <c r="B101" s="15" t="n"/>
+      <c r="B101" s="57" t="n"/>
       <c r="C101" s="14" t="n"/>
       <c r="D101" s="16" t="n"/>
       <c r="E101" s="17" t="n"/>
@@ -1979,7 +2171,7 @@
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="10" t="n"/>
-      <c r="B102" s="11" t="n"/>
+      <c r="B102" s="57" t="n"/>
       <c r="C102" s="10" t="n"/>
       <c r="D102" s="12" t="n"/>
       <c r="E102" s="13" t="n"/>
@@ -1990,7 +2182,7 @@
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="14" t="n"/>
-      <c r="B103" s="15" t="n"/>
+      <c r="B103" s="57" t="n"/>
       <c r="C103" s="14" t="n"/>
       <c r="D103" s="16" t="n"/>
       <c r="E103" s="17" t="n"/>
@@ -2001,7 +2193,7 @@
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="10" t="n"/>
-      <c r="B104" s="11" t="n"/>
+      <c r="B104" s="57" t="n"/>
       <c r="C104" s="10" t="n"/>
       <c r="D104" s="12" t="n"/>
       <c r="E104" s="13" t="n"/>
@@ -2012,7 +2204,7 @@
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="14" t="n"/>
-      <c r="B105" s="15" t="n"/>
+      <c r="B105" s="57" t="n"/>
       <c r="C105" s="14" t="n"/>
       <c r="D105" s="16" t="n"/>
       <c r="E105" s="17" t="n"/>
@@ -2023,7 +2215,7 @@
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="10" t="n"/>
-      <c r="B106" s="11" t="n"/>
+      <c r="B106" s="57" t="n"/>
       <c r="C106" s="10" t="n"/>
       <c r="D106" s="12" t="n"/>
       <c r="E106" s="13" t="n"/>
@@ -2034,7 +2226,7 @@
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="14" t="n"/>
-      <c r="B107" s="15" t="n"/>
+      <c r="B107" s="57" t="n"/>
       <c r="C107" s="14" t="n"/>
       <c r="D107" s="16" t="n"/>
       <c r="E107" s="17" t="n"/>
@@ -2045,7 +2237,7 @@
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="10" t="n"/>
-      <c r="B108" s="11" t="n"/>
+      <c r="B108" s="57" t="n"/>
       <c r="C108" s="10" t="n"/>
       <c r="D108" s="12" t="n"/>
       <c r="E108" s="13" t="n"/>
@@ -2056,7 +2248,7 @@
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="14" t="n"/>
-      <c r="B109" s="15" t="n"/>
+      <c r="B109" s="57" t="n"/>
       <c r="C109" s="14" t="n"/>
       <c r="D109" s="16" t="n"/>
       <c r="E109" s="17" t="n"/>
@@ -2067,7 +2259,7 @@
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="10" t="n"/>
-      <c r="B110" s="11" t="n"/>
+      <c r="B110" s="57" t="n"/>
       <c r="C110" s="10" t="n"/>
       <c r="D110" s="12" t="n"/>
       <c r="E110" s="13" t="n"/>
@@ -2078,7 +2270,7 @@
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="14" t="n"/>
-      <c r="B111" s="15" t="n"/>
+      <c r="B111" s="57" t="n"/>
       <c r="C111" s="14" t="n"/>
       <c r="D111" s="16" t="n"/>
       <c r="E111" s="17" t="n"/>
@@ -2089,7 +2281,7 @@
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="10" t="n"/>
-      <c r="B112" s="11" t="n"/>
+      <c r="B112" s="57" t="n"/>
       <c r="C112" s="10" t="n"/>
       <c r="D112" s="12" t="n"/>
       <c r="E112" s="13" t="n"/>
@@ -2100,7 +2292,7 @@
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="14" t="n"/>
-      <c r="B113" s="15" t="n"/>
+      <c r="B113" s="57" t="n"/>
       <c r="C113" s="14" t="n"/>
       <c r="D113" s="16" t="n"/>
       <c r="E113" s="17" t="n"/>
@@ -2111,7 +2303,7 @@
     </row>
     <row r="114" ht="20" customHeight="1">
       <c r="A114" s="10" t="n"/>
-      <c r="B114" s="11" t="n"/>
+      <c r="B114" s="57" t="n"/>
       <c r="C114" s="10" t="n"/>
       <c r="D114" s="12" t="n"/>
       <c r="E114" s="13" t="n"/>
@@ -2122,7 +2314,7 @@
     </row>
     <row r="115" ht="20" customHeight="1">
       <c r="A115" s="14" t="n"/>
-      <c r="B115" s="15" t="n"/>
+      <c r="B115" s="57" t="n"/>
       <c r="C115" s="14" t="n"/>
       <c r="D115" s="16" t="n"/>
       <c r="E115" s="17" t="n"/>
@@ -2133,7 +2325,7 @@
     </row>
     <row r="116" ht="20" customHeight="1">
       <c r="A116" s="10" t="n"/>
-      <c r="B116" s="11" t="n"/>
+      <c r="B116" s="57" t="n"/>
       <c r="C116" s="10" t="n"/>
       <c r="D116" s="12" t="n"/>
       <c r="E116" s="13" t="n"/>
@@ -2144,7 +2336,7 @@
     </row>
     <row r="117" ht="20" customHeight="1">
       <c r="A117" s="14" t="n"/>
-      <c r="B117" s="15" t="n"/>
+      <c r="B117" s="57" t="n"/>
       <c r="C117" s="14" t="n"/>
       <c r="D117" s="16" t="n"/>
       <c r="E117" s="17" t="n"/>
@@ -2155,7 +2347,7 @@
     </row>
     <row r="118" ht="20" customHeight="1">
       <c r="A118" s="10" t="n"/>
-      <c r="B118" s="11" t="n"/>
+      <c r="B118" s="57" t="n"/>
       <c r="C118" s="10" t="n"/>
       <c r="D118" s="12" t="n"/>
       <c r="E118" s="13" t="n"/>
@@ -2166,7 +2358,7 @@
     </row>
     <row r="119" ht="20" customHeight="1">
       <c r="A119" s="14" t="n"/>
-      <c r="B119" s="15" t="n"/>
+      <c r="B119" s="57" t="n"/>
       <c r="C119" s="14" t="n"/>
       <c r="D119" s="16" t="n"/>
       <c r="E119" s="17" t="n"/>
@@ -2177,7 +2369,7 @@
     </row>
     <row r="120" ht="20" customHeight="1">
       <c r="A120" s="10" t="n"/>
-      <c r="B120" s="11" t="n"/>
+      <c r="B120" s="57" t="n"/>
       <c r="C120" s="10" t="n"/>
       <c r="D120" s="12" t="n"/>
       <c r="E120" s="13" t="n"/>
@@ -2188,7 +2380,7 @@
     </row>
     <row r="121" ht="20" customHeight="1">
       <c r="A121" s="14" t="n"/>
-      <c r="B121" s="15" t="n"/>
+      <c r="B121" s="57" t="n"/>
       <c r="C121" s="14" t="n"/>
       <c r="D121" s="16" t="n"/>
       <c r="E121" s="17" t="n"/>
@@ -2199,7 +2391,7 @@
     </row>
     <row r="122" ht="20" customHeight="1">
       <c r="A122" s="10" t="n"/>
-      <c r="B122" s="11" t="n"/>
+      <c r="B122" s="57" t="n"/>
       <c r="C122" s="10" t="n"/>
       <c r="D122" s="12" t="n"/>
       <c r="E122" s="13" t="n"/>
@@ -2210,7 +2402,7 @@
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="14" t="n"/>
-      <c r="B123" s="15" t="n"/>
+      <c r="B123" s="57" t="n"/>
       <c r="C123" s="14" t="n"/>
       <c r="D123" s="16" t="n"/>
       <c r="E123" s="17" t="n"/>
@@ -2221,7 +2413,7 @@
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124" s="10" t="n"/>
-      <c r="B124" s="11" t="n"/>
+      <c r="B124" s="57" t="n"/>
       <c r="C124" s="10" t="n"/>
       <c r="D124" s="12" t="n"/>
       <c r="E124" s="13" t="n"/>
@@ -2232,7 +2424,7 @@
     </row>
     <row r="125" ht="20" customHeight="1">
       <c r="A125" s="14" t="n"/>
-      <c r="B125" s="15" t="n"/>
+      <c r="B125" s="57" t="n"/>
       <c r="C125" s="14" t="n"/>
       <c r="D125" s="16" t="n"/>
       <c r="E125" s="17" t="n"/>
@@ -2243,7 +2435,7 @@
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126" s="10" t="n"/>
-      <c r="B126" s="11" t="n"/>
+      <c r="B126" s="57" t="n"/>
       <c r="C126" s="10" t="n"/>
       <c r="D126" s="12" t="n"/>
       <c r="E126" s="13" t="n"/>
@@ -2254,7 +2446,7 @@
     </row>
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="14" t="n"/>
-      <c r="B127" s="15" t="n"/>
+      <c r="B127" s="57" t="n"/>
       <c r="C127" s="14" t="n"/>
       <c r="D127" s="16" t="n"/>
       <c r="E127" s="17" t="n"/>
@@ -2265,7 +2457,7 @@
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128" s="10" t="n"/>
-      <c r="B128" s="11" t="n"/>
+      <c r="B128" s="57" t="n"/>
       <c r="C128" s="10" t="n"/>
       <c r="D128" s="12" t="n"/>
       <c r="E128" s="13" t="n"/>
@@ -2276,7 +2468,7 @@
     </row>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="14" t="n"/>
-      <c r="B129" s="15" t="n"/>
+      <c r="B129" s="57" t="n"/>
       <c r="C129" s="14" t="n"/>
       <c r="D129" s="16" t="n"/>
       <c r="E129" s="17" t="n"/>
@@ -2287,7 +2479,7 @@
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="10" t="n"/>
-      <c r="B130" s="11" t="n"/>
+      <c r="B130" s="57" t="n"/>
       <c r="C130" s="10" t="n"/>
       <c r="D130" s="12" t="n"/>
       <c r="E130" s="13" t="n"/>
@@ -2298,7 +2490,7 @@
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="14" t="n"/>
-      <c r="B131" s="15" t="n"/>
+      <c r="B131" s="57" t="n"/>
       <c r="C131" s="14" t="n"/>
       <c r="D131" s="16" t="n"/>
       <c r="E131" s="17" t="n"/>
@@ -2309,7 +2501,7 @@
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="10" t="n"/>
-      <c r="B132" s="11" t="n"/>
+      <c r="B132" s="57" t="n"/>
       <c r="C132" s="10" t="n"/>
       <c r="D132" s="12" t="n"/>
       <c r="E132" s="13" t="n"/>
@@ -2320,7 +2512,7 @@
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="14" t="n"/>
-      <c r="B133" s="15" t="n"/>
+      <c r="B133" s="57" t="n"/>
       <c r="C133" s="14" t="n"/>
       <c r="D133" s="16" t="n"/>
       <c r="E133" s="17" t="n"/>
@@ -2331,7 +2523,7 @@
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="10" t="n"/>
-      <c r="B134" s="11" t="n"/>
+      <c r="B134" s="57" t="n"/>
       <c r="C134" s="10" t="n"/>
       <c r="D134" s="12" t="n"/>
       <c r="E134" s="13" t="n"/>
@@ -2342,7 +2534,7 @@
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="14" t="n"/>
-      <c r="B135" s="15" t="n"/>
+      <c r="B135" s="57" t="n"/>
       <c r="C135" s="14" t="n"/>
       <c r="D135" s="16" t="n"/>
       <c r="E135" s="17" t="n"/>
@@ -2353,7 +2545,7 @@
     </row>
     <row r="136" ht="20" customHeight="1">
       <c r="A136" s="10" t="n"/>
-      <c r="B136" s="11" t="n"/>
+      <c r="B136" s="57" t="n"/>
       <c r="C136" s="10" t="n"/>
       <c r="D136" s="12" t="n"/>
       <c r="E136" s="13" t="n"/>
@@ -2364,7 +2556,7 @@
     </row>
     <row r="137" ht="20" customHeight="1">
       <c r="A137" s="14" t="n"/>
-      <c r="B137" s="15" t="n"/>
+      <c r="B137" s="57" t="n"/>
       <c r="C137" s="14" t="n"/>
       <c r="D137" s="16" t="n"/>
       <c r="E137" s="17" t="n"/>
@@ -2375,7 +2567,7 @@
     </row>
     <row r="138" ht="20" customHeight="1">
       <c r="A138" s="10" t="n"/>
-      <c r="B138" s="11" t="n"/>
+      <c r="B138" s="57" t="n"/>
       <c r="C138" s="10" t="n"/>
       <c r="D138" s="12" t="n"/>
       <c r="E138" s="13" t="n"/>
@@ -2386,7 +2578,7 @@
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="14" t="n"/>
-      <c r="B139" s="15" t="n"/>
+      <c r="B139" s="57" t="n"/>
       <c r="C139" s="14" t="n"/>
       <c r="D139" s="16" t="n"/>
       <c r="E139" s="17" t="n"/>
@@ -2397,7 +2589,7 @@
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="10" t="n"/>
-      <c r="B140" s="11" t="n"/>
+      <c r="B140" s="57" t="n"/>
       <c r="C140" s="10" t="n"/>
       <c r="D140" s="12" t="n"/>
       <c r="E140" s="13" t="n"/>
@@ -2408,7 +2600,7 @@
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="14" t="n"/>
-      <c r="B141" s="15" t="n"/>
+      <c r="B141" s="57" t="n"/>
       <c r="C141" s="14" t="n"/>
       <c r="D141" s="16" t="n"/>
       <c r="E141" s="17" t="n"/>
@@ -2419,7 +2611,7 @@
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="10" t="n"/>
-      <c r="B142" s="11" t="n"/>
+      <c r="B142" s="57" t="n"/>
       <c r="C142" s="10" t="n"/>
       <c r="D142" s="12" t="n"/>
       <c r="E142" s="13" t="n"/>
@@ -2430,7 +2622,7 @@
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="14" t="n"/>
-      <c r="B143" s="15" t="n"/>
+      <c r="B143" s="57" t="n"/>
       <c r="C143" s="14" t="n"/>
       <c r="D143" s="16" t="n"/>
       <c r="E143" s="17" t="n"/>
@@ -2441,7 +2633,7 @@
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="10" t="n"/>
-      <c r="B144" s="11" t="n"/>
+      <c r="B144" s="57" t="n"/>
       <c r="C144" s="10" t="n"/>
       <c r="D144" s="12" t="n"/>
       <c r="E144" s="13" t="n"/>
@@ -2452,7 +2644,7 @@
     </row>
     <row r="145" ht="20" customHeight="1">
       <c r="A145" s="14" t="n"/>
-      <c r="B145" s="15" t="n"/>
+      <c r="B145" s="57" t="n"/>
       <c r="C145" s="14" t="n"/>
       <c r="D145" s="16" t="n"/>
       <c r="E145" s="17" t="n"/>
@@ -2463,7 +2655,7 @@
     </row>
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="10" t="n"/>
-      <c r="B146" s="11" t="n"/>
+      <c r="B146" s="57" t="n"/>
       <c r="C146" s="10" t="n"/>
       <c r="D146" s="12" t="n"/>
       <c r="E146" s="13" t="n"/>
@@ -2474,7 +2666,7 @@
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="14" t="n"/>
-      <c r="B147" s="15" t="n"/>
+      <c r="B147" s="57" t="n"/>
       <c r="C147" s="14" t="n"/>
       <c r="D147" s="16" t="n"/>
       <c r="E147" s="17" t="n"/>
@@ -2485,7 +2677,7 @@
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="10" t="n"/>
-      <c r="B148" s="11" t="n"/>
+      <c r="B148" s="57" t="n"/>
       <c r="C148" s="10" t="n"/>
       <c r="D148" s="12" t="n"/>
       <c r="E148" s="13" t="n"/>
@@ -2496,7 +2688,7 @@
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="14" t="n"/>
-      <c r="B149" s="15" t="n"/>
+      <c r="B149" s="57" t="n"/>
       <c r="C149" s="14" t="n"/>
       <c r="D149" s="16" t="n"/>
       <c r="E149" s="17" t="n"/>
@@ -2507,7 +2699,7 @@
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="10" t="n"/>
-      <c r="B150" s="11" t="n"/>
+      <c r="B150" s="57" t="n"/>
       <c r="C150" s="10" t="n"/>
       <c r="D150" s="12" t="n"/>
       <c r="E150" s="13" t="n"/>
@@ -2518,7 +2710,7 @@
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="14" t="n"/>
-      <c r="B151" s="15" t="n"/>
+      <c r="B151" s="57" t="n"/>
       <c r="C151" s="14" t="n"/>
       <c r="D151" s="16" t="n"/>
       <c r="E151" s="17" t="n"/>
@@ -2529,7 +2721,7 @@
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="10" t="n"/>
-      <c r="B152" s="11" t="n"/>
+      <c r="B152" s="57" t="n"/>
       <c r="C152" s="10" t="n"/>
       <c r="D152" s="12" t="n"/>
       <c r="E152" s="13" t="n"/>
@@ -2540,7 +2732,7 @@
     </row>
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="14" t="n"/>
-      <c r="B153" s="15" t="n"/>
+      <c r="B153" s="57" t="n"/>
       <c r="C153" s="14" t="n"/>
       <c r="D153" s="16" t="n"/>
       <c r="E153" s="17" t="n"/>
@@ -2551,7 +2743,7 @@
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="10" t="n"/>
-      <c r="B154" s="11" t="n"/>
+      <c r="B154" s="57" t="n"/>
       <c r="C154" s="10" t="n"/>
       <c r="D154" s="12" t="n"/>
       <c r="E154" s="13" t="n"/>
@@ -2562,7 +2754,7 @@
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="14" t="n"/>
-      <c r="B155" s="15" t="n"/>
+      <c r="B155" s="57" t="n"/>
       <c r="C155" s="14" t="n"/>
       <c r="D155" s="16" t="n"/>
       <c r="E155" s="17" t="n"/>
@@ -2573,7 +2765,7 @@
     </row>
     <row r="156" ht="20" customHeight="1">
       <c r="A156" s="10" t="n"/>
-      <c r="B156" s="11" t="n"/>
+      <c r="B156" s="57" t="n"/>
       <c r="C156" s="10" t="n"/>
       <c r="D156" s="12" t="n"/>
       <c r="E156" s="13" t="n"/>
@@ -2584,7 +2776,7 @@
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="14" t="n"/>
-      <c r="B157" s="15" t="n"/>
+      <c r="B157" s="57" t="n"/>
       <c r="C157" s="14" t="n"/>
       <c r="D157" s="16" t="n"/>
       <c r="E157" s="17" t="n"/>
@@ -2595,7 +2787,7 @@
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="10" t="n"/>
-      <c r="B158" s="11" t="n"/>
+      <c r="B158" s="57" t="n"/>
       <c r="C158" s="10" t="n"/>
       <c r="D158" s="12" t="n"/>
       <c r="E158" s="13" t="n"/>
@@ -2606,7 +2798,7 @@
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="14" t="n"/>
-      <c r="B159" s="15" t="n"/>
+      <c r="B159" s="57" t="n"/>
       <c r="C159" s="14" t="n"/>
       <c r="D159" s="16" t="n"/>
       <c r="E159" s="17" t="n"/>
@@ -2617,7 +2809,7 @@
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="10" t="n"/>
-      <c r="B160" s="11" t="n"/>
+      <c r="B160" s="57" t="n"/>
       <c r="C160" s="10" t="n"/>
       <c r="D160" s="12" t="n"/>
       <c r="E160" s="13" t="n"/>
@@ -2628,7 +2820,7 @@
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="14" t="n"/>
-      <c r="B161" s="15" t="n"/>
+      <c r="B161" s="57" t="n"/>
       <c r="C161" s="14" t="n"/>
       <c r="D161" s="16" t="n"/>
       <c r="E161" s="17" t="n"/>
@@ -2639,7 +2831,7 @@
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="10" t="n"/>
-      <c r="B162" s="11" t="n"/>
+      <c r="B162" s="57" t="n"/>
       <c r="C162" s="10" t="n"/>
       <c r="D162" s="12" t="n"/>
       <c r="E162" s="13" t="n"/>
@@ -2650,7 +2842,7 @@
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="14" t="n"/>
-      <c r="B163" s="15" t="n"/>
+      <c r="B163" s="57" t="n"/>
       <c r="C163" s="14" t="n"/>
       <c r="D163" s="16" t="n"/>
       <c r="E163" s="17" t="n"/>
@@ -2661,7 +2853,7 @@
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="10" t="n"/>
-      <c r="B164" s="11" t="n"/>
+      <c r="B164" s="57" t="n"/>
       <c r="C164" s="10" t="n"/>
       <c r="D164" s="12" t="n"/>
       <c r="E164" s="13" t="n"/>
@@ -2672,7 +2864,7 @@
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="14" t="n"/>
-      <c r="B165" s="15" t="n"/>
+      <c r="B165" s="57" t="n"/>
       <c r="C165" s="14" t="n"/>
       <c r="D165" s="16" t="n"/>
       <c r="E165" s="17" t="n"/>
@@ -2683,7 +2875,7 @@
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="10" t="n"/>
-      <c r="B166" s="11" t="n"/>
+      <c r="B166" s="57" t="n"/>
       <c r="C166" s="10" t="n"/>
       <c r="D166" s="12" t="n"/>
       <c r="E166" s="13" t="n"/>
@@ -2694,7 +2886,7 @@
     </row>
     <row r="167" ht="20" customHeight="1">
       <c r="A167" s="14" t="n"/>
-      <c r="B167" s="15" t="n"/>
+      <c r="B167" s="57" t="n"/>
       <c r="C167" s="14" t="n"/>
       <c r="D167" s="16" t="n"/>
       <c r="E167" s="17" t="n"/>
@@ -2705,7 +2897,7 @@
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="10" t="n"/>
-      <c r="B168" s="11" t="n"/>
+      <c r="B168" s="57" t="n"/>
       <c r="C168" s="10" t="n"/>
       <c r="D168" s="12" t="n"/>
       <c r="E168" s="13" t="n"/>
@@ -2716,7 +2908,7 @@
     </row>
     <row r="169" ht="20" customHeight="1">
       <c r="A169" s="14" t="n"/>
-      <c r="B169" s="15" t="n"/>
+      <c r="B169" s="57" t="n"/>
       <c r="C169" s="14" t="n"/>
       <c r="D169" s="16" t="n"/>
       <c r="E169" s="17" t="n"/>
@@ -2727,7 +2919,7 @@
     </row>
     <row r="170" ht="20" customHeight="1">
       <c r="A170" s="10" t="n"/>
-      <c r="B170" s="11" t="n"/>
+      <c r="B170" s="57" t="n"/>
       <c r="C170" s="10" t="n"/>
       <c r="D170" s="12" t="n"/>
       <c r="E170" s="13" t="n"/>
@@ -2738,7 +2930,7 @@
     </row>
     <row r="171" ht="20" customHeight="1">
       <c r="A171" s="14" t="n"/>
-      <c r="B171" s="15" t="n"/>
+      <c r="B171" s="57" t="n"/>
       <c r="C171" s="14" t="n"/>
       <c r="D171" s="16" t="n"/>
       <c r="E171" s="17" t="n"/>
@@ -2749,7 +2941,7 @@
     </row>
     <row r="172" ht="20" customHeight="1">
       <c r="A172" s="10" t="n"/>
-      <c r="B172" s="11" t="n"/>
+      <c r="B172" s="57" t="n"/>
       <c r="C172" s="10" t="n"/>
       <c r="D172" s="12" t="n"/>
       <c r="E172" s="13" t="n"/>
@@ -2760,7 +2952,7 @@
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="14" t="n"/>
-      <c r="B173" s="15" t="n"/>
+      <c r="B173" s="57" t="n"/>
       <c r="C173" s="14" t="n"/>
       <c r="D173" s="16" t="n"/>
       <c r="E173" s="17" t="n"/>
@@ -2771,7 +2963,7 @@
     </row>
     <row r="174" ht="20" customHeight="1">
       <c r="A174" s="10" t="n"/>
-      <c r="B174" s="11" t="n"/>
+      <c r="B174" s="57" t="n"/>
       <c r="C174" s="10" t="n"/>
       <c r="D174" s="12" t="n"/>
       <c r="E174" s="13" t="n"/>
@@ -2782,7 +2974,7 @@
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="14" t="n"/>
-      <c r="B175" s="15" t="n"/>
+      <c r="B175" s="57" t="n"/>
       <c r="C175" s="14" t="n"/>
       <c r="D175" s="16" t="n"/>
       <c r="E175" s="17" t="n"/>
@@ -2793,7 +2985,7 @@
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="A176" s="10" t="n"/>
-      <c r="B176" s="11" t="n"/>
+      <c r="B176" s="57" t="n"/>
       <c r="C176" s="10" t="n"/>
       <c r="D176" s="12" t="n"/>
       <c r="E176" s="13" t="n"/>
@@ -2804,7 +2996,7 @@
     </row>
     <row r="177" ht="20" customHeight="1">
       <c r="A177" s="14" t="n"/>
-      <c r="B177" s="15" t="n"/>
+      <c r="B177" s="57" t="n"/>
       <c r="C177" s="14" t="n"/>
       <c r="D177" s="16" t="n"/>
       <c r="E177" s="17" t="n"/>
@@ -2815,7 +3007,7 @@
     </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="10" t="n"/>
-      <c r="B178" s="11" t="n"/>
+      <c r="B178" s="57" t="n"/>
       <c r="C178" s="10" t="n"/>
       <c r="D178" s="12" t="n"/>
       <c r="E178" s="13" t="n"/>
@@ -2826,7 +3018,7 @@
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="14" t="n"/>
-      <c r="B179" s="15" t="n"/>
+      <c r="B179" s="57" t="n"/>
       <c r="C179" s="14" t="n"/>
       <c r="D179" s="16" t="n"/>
       <c r="E179" s="17" t="n"/>
@@ -2837,7 +3029,7 @@
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="10" t="n"/>
-      <c r="B180" s="11" t="n"/>
+      <c r="B180" s="57" t="n"/>
       <c r="C180" s="10" t="n"/>
       <c r="D180" s="12" t="n"/>
       <c r="E180" s="13" t="n"/>
@@ -2848,7 +3040,7 @@
     </row>
     <row r="181" ht="20" customHeight="1">
       <c r="A181" s="14" t="n"/>
-      <c r="B181" s="15" t="n"/>
+      <c r="B181" s="57" t="n"/>
       <c r="C181" s="14" t="n"/>
       <c r="D181" s="16" t="n"/>
       <c r="E181" s="17" t="n"/>
@@ -2859,7 +3051,7 @@
     </row>
     <row r="182" ht="20" customHeight="1">
       <c r="A182" s="10" t="n"/>
-      <c r="B182" s="11" t="n"/>
+      <c r="B182" s="57" t="n"/>
       <c r="C182" s="10" t="n"/>
       <c r="D182" s="12" t="n"/>
       <c r="E182" s="13" t="n"/>
@@ -2870,7 +3062,7 @@
     </row>
     <row r="183" ht="20" customHeight="1">
       <c r="A183" s="14" t="n"/>
-      <c r="B183" s="15" t="n"/>
+      <c r="B183" s="57" t="n"/>
       <c r="C183" s="14" t="n"/>
       <c r="D183" s="16" t="n"/>
       <c r="E183" s="17" t="n"/>
@@ -2881,7 +3073,7 @@
     </row>
     <row r="184" ht="20" customHeight="1">
       <c r="A184" s="10" t="n"/>
-      <c r="B184" s="11" t="n"/>
+      <c r="B184" s="57" t="n"/>
       <c r="C184" s="10" t="n"/>
       <c r="D184" s="12" t="n"/>
       <c r="E184" s="13" t="n"/>
@@ -2892,7 +3084,7 @@
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="14" t="n"/>
-      <c r="B185" s="15" t="n"/>
+      <c r="B185" s="57" t="n"/>
       <c r="C185" s="14" t="n"/>
       <c r="D185" s="16" t="n"/>
       <c r="E185" s="17" t="n"/>
@@ -2903,7 +3095,7 @@
     </row>
     <row r="186" ht="20" customHeight="1">
       <c r="A186" s="10" t="n"/>
-      <c r="B186" s="11" t="n"/>
+      <c r="B186" s="57" t="n"/>
       <c r="C186" s="10" t="n"/>
       <c r="D186" s="12" t="n"/>
       <c r="E186" s="13" t="n"/>
@@ -2914,7 +3106,7 @@
     </row>
     <row r="187" ht="20" customHeight="1">
       <c r="A187" s="14" t="n"/>
-      <c r="B187" s="15" t="n"/>
+      <c r="B187" s="57" t="n"/>
       <c r="C187" s="14" t="n"/>
       <c r="D187" s="16" t="n"/>
       <c r="E187" s="17" t="n"/>
@@ -2925,7 +3117,7 @@
     </row>
     <row r="188" ht="20" customHeight="1">
       <c r="A188" s="10" t="n"/>
-      <c r="B188" s="11" t="n"/>
+      <c r="B188" s="57" t="n"/>
       <c r="C188" s="10" t="n"/>
       <c r="D188" s="12" t="n"/>
       <c r="E188" s="13" t="n"/>
@@ -2936,7 +3128,7 @@
     </row>
     <row r="189" ht="20" customHeight="1">
       <c r="A189" s="14" t="n"/>
-      <c r="B189" s="15" t="n"/>
+      <c r="B189" s="57" t="n"/>
       <c r="C189" s="14" t="n"/>
       <c r="D189" s="16" t="n"/>
       <c r="E189" s="17" t="n"/>
@@ -2947,7 +3139,7 @@
     </row>
     <row r="190" ht="20" customHeight="1">
       <c r="A190" s="10" t="n"/>
-      <c r="B190" s="11" t="n"/>
+      <c r="B190" s="57" t="n"/>
       <c r="C190" s="10" t="n"/>
       <c r="D190" s="12" t="n"/>
       <c r="E190" s="13" t="n"/>
@@ -2958,7 +3150,7 @@
     </row>
     <row r="191" ht="20" customHeight="1">
       <c r="A191" s="14" t="n"/>
-      <c r="B191" s="15" t="n"/>
+      <c r="B191" s="57" t="n"/>
       <c r="C191" s="14" t="n"/>
       <c r="D191" s="16" t="n"/>
       <c r="E191" s="17" t="n"/>
@@ -2969,7 +3161,7 @@
     </row>
     <row r="192" ht="20" customHeight="1">
       <c r="A192" s="10" t="n"/>
-      <c r="B192" s="11" t="n"/>
+      <c r="B192" s="57" t="n"/>
       <c r="C192" s="10" t="n"/>
       <c r="D192" s="12" t="n"/>
       <c r="E192" s="13" t="n"/>
@@ -2980,7 +3172,7 @@
     </row>
     <row r="193" ht="20" customHeight="1">
       <c r="A193" s="14" t="n"/>
-      <c r="B193" s="15" t="n"/>
+      <c r="B193" s="57" t="n"/>
       <c r="C193" s="14" t="n"/>
       <c r="D193" s="16" t="n"/>
       <c r="E193" s="17" t="n"/>
@@ -2991,7 +3183,7 @@
     </row>
     <row r="194" ht="20" customHeight="1">
       <c r="A194" s="10" t="n"/>
-      <c r="B194" s="11" t="n"/>
+      <c r="B194" s="57" t="n"/>
       <c r="C194" s="10" t="n"/>
       <c r="D194" s="12" t="n"/>
       <c r="E194" s="13" t="n"/>
@@ -3002,7 +3194,7 @@
     </row>
     <row r="195" ht="20" customHeight="1">
       <c r="A195" s="14" t="n"/>
-      <c r="B195" s="15" t="n"/>
+      <c r="B195" s="57" t="n"/>
       <c r="C195" s="14" t="n"/>
       <c r="D195" s="16" t="n"/>
       <c r="E195" s="17" t="n"/>
@@ -3013,7 +3205,7 @@
     </row>
     <row r="196" ht="20" customHeight="1">
       <c r="A196" s="10" t="n"/>
-      <c r="B196" s="11" t="n"/>
+      <c r="B196" s="57" t="n"/>
       <c r="C196" s="10" t="n"/>
       <c r="D196" s="12" t="n"/>
       <c r="E196" s="13" t="n"/>
@@ -3024,7 +3216,7 @@
     </row>
     <row r="197" ht="20" customHeight="1">
       <c r="A197" s="14" t="n"/>
-      <c r="B197" s="15" t="n"/>
+      <c r="B197" s="57" t="n"/>
       <c r="C197" s="14" t="n"/>
       <c r="D197" s="16" t="n"/>
       <c r="E197" s="17" t="n"/>
@@ -3035,7 +3227,7 @@
     </row>
     <row r="198" ht="20" customHeight="1">
       <c r="A198" s="10" t="n"/>
-      <c r="B198" s="11" t="n"/>
+      <c r="B198" s="57" t="n"/>
       <c r="C198" s="10" t="n"/>
       <c r="D198" s="12" t="n"/>
       <c r="E198" s="13" t="n"/>
@@ -3046,7 +3238,7 @@
     </row>
     <row r="199" ht="20" customHeight="1">
       <c r="A199" s="14" t="n"/>
-      <c r="B199" s="15" t="n"/>
+      <c r="B199" s="57" t="n"/>
       <c r="C199" s="14" t="n"/>
       <c r="D199" s="16" t="n"/>
       <c r="E199" s="17" t="n"/>
@@ -3057,7 +3249,7 @@
     </row>
     <row r="200" ht="20" customHeight="1">
       <c r="A200" s="10" t="n"/>
-      <c r="B200" s="11" t="n"/>
+      <c r="B200" s="57" t="n"/>
       <c r="C200" s="10" t="n"/>
       <c r="D200" s="12" t="n"/>
       <c r="E200" s="13" t="n"/>
@@ -3068,7 +3260,7 @@
     </row>
     <row r="201" ht="20" customHeight="1">
       <c r="A201" s="14" t="n"/>
-      <c r="B201" s="15" t="n"/>
+      <c r="B201" s="57" t="n"/>
       <c r="C201" s="14" t="n"/>
       <c r="D201" s="16" t="n"/>
       <c r="E201" s="17" t="n"/>
@@ -3079,7 +3271,7 @@
     </row>
     <row r="202" ht="20" customHeight="1">
       <c r="A202" s="10" t="n"/>
-      <c r="B202" s="11" t="n"/>
+      <c r="B202" s="57" t="n"/>
       <c r="C202" s="10" t="n"/>
       <c r="D202" s="12" t="n"/>
       <c r="E202" s="13" t="n"/>
@@ -3090,7 +3282,7 @@
     </row>
     <row r="203" ht="20" customHeight="1">
       <c r="A203" s="14" t="n"/>
-      <c r="B203" s="15" t="n"/>
+      <c r="B203" s="57" t="n"/>
       <c r="C203" s="14" t="n"/>
       <c r="D203" s="16" t="n"/>
       <c r="E203" s="17" t="n"/>
@@ -3101,7 +3293,7 @@
     </row>
     <row r="204" ht="20" customHeight="1">
       <c r="A204" s="10" t="n"/>
-      <c r="B204" s="11" t="n"/>
+      <c r="B204" s="57" t="n"/>
       <c r="C204" s="10" t="n"/>
       <c r="D204" s="12" t="n"/>
       <c r="E204" s="13" t="n"/>
@@ -3112,7 +3304,7 @@
     </row>
     <row r="205" ht="20" customHeight="1">
       <c r="A205" s="14" t="n"/>
-      <c r="B205" s="15" t="n"/>
+      <c r="B205" s="57" t="n"/>
       <c r="C205" s="14" t="n"/>
       <c r="D205" s="16" t="n"/>
       <c r="E205" s="17" t="n"/>
@@ -3123,7 +3315,7 @@
     </row>
     <row r="206" ht="20" customHeight="1">
       <c r="A206" s="10" t="n"/>
-      <c r="B206" s="11" t="n"/>
+      <c r="B206" s="57" t="n"/>
       <c r="C206" s="10" t="n"/>
       <c r="D206" s="12" t="n"/>
       <c r="E206" s="13" t="n"/>
@@ -3178,6 +3370,15 @@
           <t>EVENTS MASTER — All Team Events &amp; Costs</t>
         </is>
       </c>
+      <c r="B1" s="53" t="n"/>
+      <c r="C1" s="53" t="n"/>
+      <c r="D1" s="53" t="n"/>
+      <c r="E1" s="53" t="n"/>
+      <c r="F1" s="53" t="n"/>
+      <c r="G1" s="53" t="n"/>
+      <c r="H1" s="53" t="n"/>
+      <c r="I1" s="53" t="n"/>
+      <c r="J1" s="54" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
@@ -9630,10 +9831,15 @@
           <t>ATTENDANCE TRACKER</t>
         </is>
       </c>
+      <c r="B1" s="53" t="n"/>
+      <c r="C1" s="53" t="n"/>
+      <c r="D1" s="53" t="n"/>
+      <c r="E1" s="53" t="n"/>
+      <c r="F1" s="54" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1"/>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="42" t="inlineStr">
         <is>
           <t>← Player Name</t>
         </is>
@@ -9829,215 +10035,215 @@
       <c r="AZ6" s="28" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t>Total Attendees →</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr"/>
       <c r="C7" s="30">
-        <f>COUNTIF(C10:C209,"Y")+COUNTIF(C10:C209,"1")</f>
+        <f>COUNTIF(C10:C209,"1")</f>
         <v/>
       </c>
       <c r="D7" s="30">
-        <f>COUNTIF(D10:D209,"Y")+COUNTIF(D10:D209,"1")</f>
+        <f>COUNTIF(D10:D209,"1")</f>
         <v/>
       </c>
       <c r="E7" s="30">
-        <f>COUNTIF(E10:E209,"Y")+COUNTIF(E10:E209,"1")</f>
+        <f>COUNTIF(E10:E209,"1")</f>
         <v/>
       </c>
       <c r="F7" s="30">
-        <f>COUNTIF(F10:F209,"Y")+COUNTIF(F10:F209,"1")</f>
+        <f>COUNTIF(F10:F209,"1")</f>
         <v/>
       </c>
       <c r="G7" s="30">
-        <f>COUNTIF(G10:G209,"Y")+COUNTIF(G10:G209,"1")</f>
+        <f>COUNTIF(G10:G209,"1")</f>
         <v/>
       </c>
       <c r="H7" s="30">
-        <f>COUNTIF(H10:H209,"Y")+COUNTIF(H10:H209,"1")</f>
+        <f>COUNTIF(H10:H209,"1")</f>
         <v/>
       </c>
       <c r="I7" s="30">
-        <f>COUNTIF(I10:I209,"Y")+COUNTIF(I10:I209,"1")</f>
+        <f>COUNTIF(I10:I209,"1")</f>
         <v/>
       </c>
       <c r="J7" s="30">
-        <f>COUNTIF(J10:J209,"Y")+COUNTIF(J10:J209,"1")</f>
+        <f>COUNTIF(J10:J209,"1")</f>
         <v/>
       </c>
       <c r="K7" s="30">
-        <f>COUNTIF(K10:K209,"Y")+COUNTIF(K10:K209,"1")</f>
+        <f>COUNTIF(K10:K209,"1")</f>
         <v/>
       </c>
       <c r="L7" s="30">
-        <f>COUNTIF(L10:L209,"Y")+COUNTIF(L10:L209,"1")</f>
+        <f>COUNTIF(L10:L209,"1")</f>
         <v/>
       </c>
       <c r="M7" s="30">
-        <f>COUNTIF(M10:M209,"Y")+COUNTIF(M10:M209,"1")</f>
+        <f>COUNTIF(M10:M209,"1")</f>
         <v/>
       </c>
       <c r="N7" s="30">
-        <f>COUNTIF(N10:N209,"Y")+COUNTIF(N10:N209,"1")</f>
+        <f>COUNTIF(N10:N209,"1")</f>
         <v/>
       </c>
       <c r="O7" s="30">
-        <f>COUNTIF(O10:O209,"Y")+COUNTIF(O10:O209,"1")</f>
+        <f>COUNTIF(O10:O209,"1")</f>
         <v/>
       </c>
       <c r="P7" s="30">
-        <f>COUNTIF(P10:P209,"Y")+COUNTIF(P10:P209,"1")</f>
+        <f>COUNTIF(P10:P209,"1")</f>
         <v/>
       </c>
       <c r="Q7" s="30">
-        <f>COUNTIF(Q10:Q209,"Y")+COUNTIF(Q10:Q209,"1")</f>
+        <f>COUNTIF(Q10:Q209,"1")</f>
         <v/>
       </c>
       <c r="R7" s="30">
-        <f>COUNTIF(R10:R209,"Y")+COUNTIF(R10:R209,"1")</f>
+        <f>COUNTIF(R10:R209,"1")</f>
         <v/>
       </c>
       <c r="S7" s="30">
-        <f>COUNTIF(S10:S209,"Y")+COUNTIF(S10:S209,"1")</f>
+        <f>COUNTIF(S10:S209,"1")</f>
         <v/>
       </c>
       <c r="T7" s="30">
-        <f>COUNTIF(T10:T209,"Y")+COUNTIF(T10:T209,"1")</f>
+        <f>COUNTIF(T10:T209,"1")</f>
         <v/>
       </c>
       <c r="U7" s="30">
-        <f>COUNTIF(U10:U209,"Y")+COUNTIF(U10:U209,"1")</f>
+        <f>COUNTIF(U10:U209,"1")</f>
         <v/>
       </c>
       <c r="V7" s="30">
-        <f>COUNTIF(V10:V209,"Y")+COUNTIF(V10:V209,"1")</f>
+        <f>COUNTIF(V10:V209,"1")</f>
         <v/>
       </c>
       <c r="W7" s="30">
-        <f>COUNTIF(W10:W209,"Y")+COUNTIF(W10:W209,"1")</f>
+        <f>COUNTIF(W10:W209,"1")</f>
         <v/>
       </c>
       <c r="X7" s="30">
-        <f>COUNTIF(X10:X209,"Y")+COUNTIF(X10:X209,"1")</f>
+        <f>COUNTIF(X10:X209,"1")</f>
         <v/>
       </c>
       <c r="Y7" s="30">
-        <f>COUNTIF(Y10:Y209,"Y")+COUNTIF(Y10:Y209,"1")</f>
+        <f>COUNTIF(Y10:Y209,"1")</f>
         <v/>
       </c>
       <c r="Z7" s="30">
-        <f>COUNTIF(Z10:Z209,"Y")+COUNTIF(Z10:Z209,"1")</f>
+        <f>COUNTIF(Z10:Z209,"1")</f>
         <v/>
       </c>
       <c r="AA7" s="30">
-        <f>COUNTIF(AA10:AA209,"Y")+COUNTIF(AA10:AA209,"1")</f>
+        <f>COUNTIF(AA10:AA209,"1")</f>
         <v/>
       </c>
       <c r="AB7" s="30">
-        <f>COUNTIF(AB10:AB209,"Y")+COUNTIF(AB10:AB209,"1")</f>
+        <f>COUNTIF(AB10:AB209,"1")</f>
         <v/>
       </c>
       <c r="AC7" s="30">
-        <f>COUNTIF(AC10:AC209,"Y")+COUNTIF(AC10:AC209,"1")</f>
+        <f>COUNTIF(AC10:AC209,"1")</f>
         <v/>
       </c>
       <c r="AD7" s="30">
-        <f>COUNTIF(AD10:AD209,"Y")+COUNTIF(AD10:AD209,"1")</f>
+        <f>COUNTIF(AD10:AD209,"1")</f>
         <v/>
       </c>
       <c r="AE7" s="30">
-        <f>COUNTIF(AE10:AE209,"Y")+COUNTIF(AE10:AE209,"1")</f>
+        <f>COUNTIF(AE10:AE209,"1")</f>
         <v/>
       </c>
       <c r="AF7" s="30">
-        <f>COUNTIF(AF10:AF209,"Y")+COUNTIF(AF10:AF209,"1")</f>
+        <f>COUNTIF(AF10:AF209,"1")</f>
         <v/>
       </c>
       <c r="AG7" s="30">
-        <f>COUNTIF(AG10:AG209,"Y")+COUNTIF(AG10:AG209,"1")</f>
+        <f>COUNTIF(AG10:AG209,"1")</f>
         <v/>
       </c>
       <c r="AH7" s="30">
-        <f>COUNTIF(AH10:AH209,"Y")+COUNTIF(AH10:AH209,"1")</f>
+        <f>COUNTIF(AH10:AH209,"1")</f>
         <v/>
       </c>
       <c r="AI7" s="30">
-        <f>COUNTIF(AI10:AI209,"Y")+COUNTIF(AI10:AI209,"1")</f>
+        <f>COUNTIF(AI10:AI209,"1")</f>
         <v/>
       </c>
       <c r="AJ7" s="30">
-        <f>COUNTIF(AJ10:AJ209,"Y")+COUNTIF(AJ10:AJ209,"1")</f>
+        <f>COUNTIF(AJ10:AJ209,"1")</f>
         <v/>
       </c>
       <c r="AK7" s="30">
-        <f>COUNTIF(AK10:AK209,"Y")+COUNTIF(AK10:AK209,"1")</f>
+        <f>COUNTIF(AK10:AK209,"1")</f>
         <v/>
       </c>
       <c r="AL7" s="30">
-        <f>COUNTIF(AL10:AL209,"Y")+COUNTIF(AL10:AL209,"1")</f>
+        <f>COUNTIF(AL10:AL209,"1")</f>
         <v/>
       </c>
       <c r="AM7" s="30">
-        <f>COUNTIF(AM10:AM209,"Y")+COUNTIF(AM10:AM209,"1")</f>
+        <f>COUNTIF(AM10:AM209,"1")</f>
         <v/>
       </c>
       <c r="AN7" s="30">
-        <f>COUNTIF(AN10:AN209,"Y")+COUNTIF(AN10:AN209,"1")</f>
+        <f>COUNTIF(AN10:AN209,"1")</f>
         <v/>
       </c>
       <c r="AO7" s="30">
-        <f>COUNTIF(AO10:AO209,"Y")+COUNTIF(AO10:AO209,"1")</f>
+        <f>COUNTIF(AO10:AO209,"1")</f>
         <v/>
       </c>
       <c r="AP7" s="30">
-        <f>COUNTIF(AP10:AP209,"Y")+COUNTIF(AP10:AP209,"1")</f>
+        <f>COUNTIF(AP10:AP209,"1")</f>
         <v/>
       </c>
       <c r="AQ7" s="30">
-        <f>COUNTIF(AQ10:AQ209,"Y")+COUNTIF(AQ10:AQ209,"1")</f>
+        <f>COUNTIF(AQ10:AQ209,"1")</f>
         <v/>
       </c>
       <c r="AR7" s="30">
-        <f>COUNTIF(AR10:AR209,"Y")+COUNTIF(AR10:AR209,"1")</f>
+        <f>COUNTIF(AR10:AR209,"1")</f>
         <v/>
       </c>
       <c r="AS7" s="30">
-        <f>COUNTIF(AS10:AS209,"Y")+COUNTIF(AS10:AS209,"1")</f>
+        <f>COUNTIF(AS10:AS209,"1")</f>
         <v/>
       </c>
       <c r="AT7" s="30">
-        <f>COUNTIF(AT10:AT209,"Y")+COUNTIF(AT10:AT209,"1")</f>
+        <f>COUNTIF(AT10:AT209,"1")</f>
         <v/>
       </c>
       <c r="AU7" s="30">
-        <f>COUNTIF(AU10:AU209,"Y")+COUNTIF(AU10:AU209,"1")</f>
+        <f>COUNTIF(AU10:AU209,"1")</f>
         <v/>
       </c>
       <c r="AV7" s="30">
-        <f>COUNTIF(AV10:AV209,"Y")+COUNTIF(AV10:AV209,"1")</f>
+        <f>COUNTIF(AV10:AV209,"1")</f>
         <v/>
       </c>
       <c r="AW7" s="30">
-        <f>COUNTIF(AW10:AW209,"Y")+COUNTIF(AW10:AW209,"1")</f>
+        <f>COUNTIF(AW10:AW209,"1")</f>
         <v/>
       </c>
       <c r="AX7" s="30">
-        <f>COUNTIF(AX10:AX209,"Y")+COUNTIF(AX10:AX209,"1")</f>
+        <f>COUNTIF(AX10:AX209,"1")</f>
         <v/>
       </c>
       <c r="AY7" s="30">
-        <f>COUNTIF(AY10:AY209,"Y")+COUNTIF(AY10:AY209,"1")</f>
+        <f>COUNTIF(AY10:AY209,"1")</f>
         <v/>
       </c>
       <c r="AZ7" s="30">
-        <f>COUNTIF(AZ10:AZ209,"Y")+COUNTIF(AZ10:AZ209,"1")</f>
+        <f>COUNTIF(AZ10:AZ209,"1")</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>Total Cost →</t>
         </is>
@@ -10252,7 +10458,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -21295,7 +21501,7 @@
     <row r="209" ht="20" customHeight="1">
       <c r="A209" s="34" t="inlineStr">
         <is>
-          <t>Y = Attended | N = Absent | E = Excused</t>
+          <t>1 = Attended  |  0 = Absent  |  X = Exempt</t>
         </is>
       </c>
       <c r="B209" s="6" t="n"/>
@@ -21356,7 +21562,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C86 C87 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C102 C103 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C118 C119 C120 C121 C122 C123 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C134 C135 C136 C137 C138 C139 C140 C141 C142 C143 C144 C145 C146 C147 C148 C149 C150 C151 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C162 C163 C164 C165 C166 C167 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 C182 C183 C184 C185 C186 C187 C188 C189 C190 C191 C192 C193 C194 C195 C196 C197 C198 C199 C200 C201 C202 C203 C204 C205 C206 C207 C208 C209 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147 D148 D149 D150 D151 D152 D153 D154 D155 D156 D157 D158 D159 D160 D161 D162 D163 D164 D165 D166 D167 D168 D169 D170 D171 D172 D173 D174 D175 D176 D177 D178 D179 D180 D181 D182 D183 D184 D185 D186 D187 D188 D189 D190 D191 D192 D193 D194 D195 D196 D197 D198 D199 D200 D201 D202 D203 D204 D205 D206 D207 D208 D209 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E97 E98 E99 E100 E101 E102 E103 E104 E105 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E135 E136 E137 E138 E139 E140 E141 E142 E143 E144 E145 E146 E147 E148 E149 E150 E151 E152 E153 E154 E155 E156 E157 E158 E159 E160 E161 E162 E163 E164 E165 E166 E167 E168 E169 E170 E171 E172 E173 E174 E175 E176 E177 E178 E179 E180 E181 E182 E183 E184 E185 E186 E187 E188 E189 E190 E191 E192 E193 E194 E195 E196 E197 E198 E199 E200 E201 E202 E203 E204 E205 E206 E207 E208 E209 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 F48 F49 F50 F51 F52 F53 F54 F55 F56 F57 F58 F59 F60 F61 F62 F63 F64 F65 F66 F67 F68 F69 F70 F71 F72 F73 F74 F75 F76 F77 F78 F79 F80 F81 F82 F83 F84 F85 F86 F87 F88 F89 F90 F91 F92 F93 F94 F95 F96 F97 F98 F99 F100 F101 F102 F103 F104 F105 F106 F107 F108 F109 F110 F111 F112 F113 F114 F115 F116 F117 F118 F119 F120 F121 F122 F123 F124 F125 F126 F127 F128 F129 F130 F131 F132 F133 F134 F135 F136 F137 F138 F139 F140 F141 F142 F143 F144 F145 F146 F147 F148 F149 F150 F151 F152 F153 F154 F155 F156 F157 F158 F159 F160 F161 F162 F163 F164 F165 F166 F167 F168 F169 F170 F171 F172 F173 F174 F175 F176 F177 F178 F179 F180 F181 F182 F183 F184 F185 F186 F187 F188 F189 F190 F191 F192 F193 F194 F195 F196 F197 F198 F199 F200 F201 F202 F203 F204 F205 F206 F207 F208 F209 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51 G52 G53 G54 G55 G56 G57 G58 G59 G60 G61 G62 G63 G64 G65 G66 G67 G68 G69 G70 G71 G72 G73 G74 G75 G76 G77 G78 G79 G80 G81 G82 G83 G84 G85 G86 G87 G88 G89 G90 G91 G92 G93 G94 G95 G96 G97 G98 G99 G100 G101 G102 G103 G104 G105 G106 G107 G108 G109 G110 G111 G112 G113 G114 G115 G116 G117 G118 G119 G120 G121 G122 G123 G124 G125 G126 G127 G128 G129 G130 G131 G132 G133 G134 G135 G136 G137 G138 G139 G140 G141 G142 G143 G144 G145 G146 G147 G148 G149 G150 G151 G152 G153 G154 G155 G156 G157 G158 G159 G160 G161 G162 G163 G164 G165 G166 G167 G168 G169 G170 G171 G172 G173 G174 G175 G176 G177 G178 G179 G180 G181 G182 G183 G184 G185 G186 G187 G188 G189 G190 G191 G192 G193 G194 G195 G196 G197 G198 G199 G200 G201 G202 G203 G204 G205 G206 G207 G208 G209 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H182 H183 H184 H185 H186 H187 H188 H189 H190 H191 H192 H193 H194 H195 H196 H197 H198 H199 H200 H201 H202 H203 H204 H205 H206 H207 H208 H209 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 I46 I47 I48 I49 I50 I51 I52 I53 I54 I55 I56 I57 I58 I59 I60 I61 I62 I63 I64 I65 I66 I67 I68 I69 I70 I71 I72 I73 I74 I75 I76 I77 I78 I79 I80 I81 I82 I83 I84 I85 I86 I87 I88 I89 I90 I91 I92 I93 I94 I95 I96 I97 I98 I99 I100 I101 I102 I103 I104 I105 I106 I107 I108 I109 I110 I111 I112 I113 I114 I115 I116 I117 I118 I119 I120 I121 I122 I123 I124 I125 I126 I127 I128 I129 I130 I131 I132 I133 I134 I135 I136 I137 I138 I139 I140 I141 I142 I143 I144 I145 I146 I147 I148 I149 I150 I151 I152 I153 I154 I155 I156 I157 I158 I159 I160 I161 I162 I163 I164 I165 I166 I167 I168 I169 I170 I171 I172 I173 I174 I175 I176 I177 I178 I179 I180 I181 I182 I183 I184 I185 I186 I187 I188 I189 I190 I191 I192 I193 I194 I195 I196 I197 I198 I199 I200 I201 I202 I203 I204 I205 I206 I207 I208 I209 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 J46 J47 J48 J49 J50 J51 J52 J53 J54 J55 J56 J57 J58 J59 J60 J61 J62 J63 J64 J65 J66 J67 J68 J69 J70 J71 J72 J73 J74 J75 J76 J77 J78 J79 J80 J81 J82 J83 J84 J85 J86 J87 J88 J89 J90 J91 J92 J93 J94 J95 J96 J97 J98 J99 J100 J101 J102 J103 J104 J105 J106 J107 J108 J109 J110 J111 J112 J113 J114 J115 J116 J117 J118 J119 J120 J121 J122 J123 J124 J125 J126 J127 J128 J129 J130 J131 J132 J133 J134 J135 J136 J137 J138 J139 J140 J141 J142 J143 J144 J145 J146 J147 J148 J149 J150 J151 J152 J153 J154 J155 J156 J157 J158 J159 J160 J161 J162 J163 J164 J165 J166 J167 J168 J169 J170 J171 J172 J173 J174 J175 J176 J177 J178 J179 J180 J181 J182 J183 J184 J185 J186 J187 J188 J189 J190 J191 J192 J193 J194 J195 J196 J197 J198 J199 J200 J201 J202 J203 J204 J205 J206 J207 J208 J209 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 K92 K93 K94 K95 K96 K97 K98 K99 K100 K101 K102 K103 K104 K105 K106 K107 K108 K109 K110 K111 K112 K113 K114 K115 K116 K117 K118 K119 K120 K121 K122 K123 K124 K125 K126 K127 K128 K129 K130 K131 K132 K133 K134 K135 K136 K137 K138 K139 K140 K141 K142 K143 K144 K145 K146 K147 K148 K149 K150 K151 K152 K153 K154 K155 K156 K157 K158 K159 K160 K161 K162 K163 K164 K165 K166 K167 K168 K169 K170 K171 K172 K173 K174 K175 K176 K177 K178 K179 K180 K181 K182 K183 K184 K185 K186 K187 K188 K189 K190 K191 K192 K193 K194 K195 K196 K197 K198 K199 K200 K201 K202 K203 K204 K205 K206 K207 K208 K209 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 L46 L47 L48 L49 L50 L51 L52 L53 L54 L55 L56 L57 L58 L59 L60 L61 L62 L63 L64 L65 L66 L67 L68 L69 L70 L71 L72 L73 L74 L75 L76 L77 L78 L79 L80 L81 L82 L83 L84 L85 L86 L87 L88 L89 L90 L91 L92 L93 L94 L95 L96 L97 L98 L99 L100 L101 L102 L103 L104 L105 L106 L107 L108 L109 L110 L111 L112 L113 L114 L115 L116 L117 L118 L119 L120 L121 L122 L123 L124 L125 L126 L127 L128 L129 L130 L131 L132 L133 L134 L135 L136 L137 L138 L139 L140 L141 L142 L143 L144 L145 L146 L147 L148 L149 L150 L151 L152 L153 L154 L155 L156 L157 L158 L159 L160 L161 L162 L163 L164 L165 L166 L167 L168 L169 L170 L171 L172 L173 L174 L175 L176 L177 L178 L179 L180 L181 L182 L183 L184 L185 L186 L187 L188 L189 L190 L191 L192 L193 L194 L195 L196 L197 L198 L199 L200 L201 L202 L203 L204 L205 L206 L207 L208 L209 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 M41 M42 M43 M44 M45 M46 M47 M48 M49 M50 M51 M52 M53 M54 M55 M56 M57 M58 M59 M60 M61 M62 M63 M64 M65 M66 M67 M68 M69 M70 M71 M72 M73 M74 M75 M76 M77 M78 M79 M80 M81 M82 M83 M84 M85 M86 M87 M88 M89 M90 M91 M92 M93 M94 M95 M96 M97 M98 M99 M100 M101 M102 M103 M104 M105 M106 M107 M108 M109 M110 M111 M112 M113 M114 M115 M116 M117 M118 M119 M120 M121 M122 M123 M124 M125 M126 M127 M128 M129 M130 M131 M132 M133 M134 M135 M136 M137 M138 M139 M140 M141 M142 M143 M144 M145 M146 M147 M148 M149 M150 M151 M152 M153 M154 M155 M156 M157 M158 M159 M160 M161 M162 M163 M164 M165 M166 M167 M168 M169 M170 M171 M172 M173 M174 M175 M176 M177 M178 M179 M180 M181 M182 M183 M184 M185 M186 M187 M188 M189 M190 M191 M192 M193 M194 M195 M196 M197 M198 M199 M200 M201 M202 M203 M204 M205 M206 M207 M208 M209 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 N46 N47 N48 N49 N50 N51 N52 N53 N54 N55 N56 N57 N58 N59 N60 N61 N62 N63 N64 N65 N66 N67 N68 N69 N70 N71 N72 N73 N74 N75 N76 N77 N78 N79 N80 N81 N82 N83 N84 N85 N86 N87 N88 N89 N90 N91 N92 N93 N94 N95 N96 N97 N98 N99 N100 N101 N102 N103 N104 N105 N106 N107 N108 N109 N110 N111 N112 N113 N114 N115 N116 N117 N118 N119 N120 N121 N122 N123 N124 N125 N126 N127 N128 N129 N130 N131 N132 N133 N134 N135 N136 N137 N138 N139 N140 N141 N142 N143 N144 N145 N146 N147 N148 N149 N150 N151 N152 N153 N154 N155 N156 N157 N158 N159 N160 N161 N162 N163 N164 N165 N166 N167 N168 N169 N170 N171 N172 N173 N174 N175 N176 N177 N178 N179 N180 N181 N182 N183 N184 N185 N186 N187 N188 N189 N190 N191 N192 N193 N194 N195 N196 N197 N198 N199 N200 N201 N202 N203 N204 N205 N206 N207 N208 N209 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54 O55 O56 O57 O58 O59 O60 O61 O62 O63 O64 O65 O66 O67 O68 O69 O70 O71 O72 O73 O74 O75 O76 O77 O78 O79 O80 O81 O82 O83 O84 O85 O86 O87 O88 O89 O90 O91 O92 O93 O94 O95 O96 O97 O98 O99 O100 O101 O102 O103 O104 O105 O106 O107 O108 O109 O110 O111 O112 O113 O114 O115 O116 O117 O118 O119 O120 O121 O122 O123 O124 O125 O126 O127 O128 O129 O130 O131 O132 O133 O134 O135 O136 O137 O138 O139 O140 O141 O142 O143 O144 O145 O146 O147 O148 O149 O150 O151 O152 O153 O154 O155 O156 O157 O158 O159 O160 O161 O162 O163 O164 O165 O166 O167 O168 O169 O170 O171 O172 O173 O174 O175 O176 O177 O178 O179 O180 O181 O182 O183 O184 O185 O186 O187 O188 O189 O190 O191 O192 O193 O194 O195 O196 O197 O198 O199 O200 O201 O202 O203 O204 O205 O206 O207 O208 O209 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 P41 P42 P43 P44 P45 P46 P47 P48 P49 P50 P51 P52 P53 P54 P55 P56 P57 P58 P59 P60 P61 P62 P63 P64 P65 P66 P67 P68 P69 P70 P71 P72 P73 P74 P75 P76 P77 P78 P79 P80 P81 P82 P83 P84 P85 P86 P87 P88 P89 P90 P91 P92 P93 P94 P95 P96 P97 P98 P99 P100 P101 P102 P103 P104 P105 P106 P107 P108 P109 P110 P111 P112 P113 P114 P115 P116 P117 P118 P119 P120 P121 P122 P123 P124 P125 P126 P127 P128 P129 P130 P131 P132 P133 P134 P135 P136 P137 P138 P139 P140 P141 P142 P143 P144 P145 P146 P147 P148 P149 P150 P151 P152 P153 P154 P155 P156 P157 P158 P159 P160 P161 P162 P163 P164 P165 P166 P167 P168 P169 P170 P171 P172 P173 P174 P175 P176 P177 P178 P179 P180 P181 P182 P183 P184 P185 P186 P187 P188 P189 P190 P191 P192 P193 P194 P195 P196 P197 P198 P199 P200 P201 P202 P203 P204 P205 P206 P207 P208 P209 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 Q46 Q47 Q48 Q49 Q50 Q51 Q52 Q53 Q54 Q55 Q56 Q57 Q58 Q59 Q60 Q61 Q62 Q63 Q64 Q65 Q66 Q67 Q68 Q69 Q70 Q71 Q72 Q73 Q74 Q75 Q76 Q77 Q78 Q79 Q80 Q81 Q82 Q83 Q84 Q85 Q86 Q87 Q88 Q89 Q90 Q91 Q92 Q93 Q94 Q95 Q96 Q97 Q98 Q99 Q100 Q101 Q102 Q103 Q104 Q105 Q106 Q107 Q108 Q109 Q110 Q111 Q112 Q113 Q114 Q115 Q116 Q117 Q118 Q119 Q120 Q121 Q122 Q123 Q124 Q125 Q126 Q127 Q128 Q129 Q130 Q131 Q132 Q133 Q134 Q135 Q136 Q137 Q138 Q139 Q140 Q141 Q142 Q143 Q144 Q145 Q146 Q147 Q148 Q149 Q150 Q151 Q152 Q153 Q154 Q155 Q156 Q157 Q158 Q159 Q160 Q161 Q162 Q163 Q164 Q165 Q166 Q167 Q168 Q169 Q170 Q171 Q172 Q173 Q174 Q175 Q176 Q177 Q178 Q179 Q180 Q181 Q182 Q183 Q184 Q185 Q186 Q187 Q188 Q189 Q190 Q191 Q192 Q193 Q194 Q195 Q196 Q197 Q198 Q199 Q200 Q201 Q202 Q203 Q204 Q205 Q206 Q207 Q208 Q209 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 R46 R47 R48 R49 R50 R51 R52 R53 R54 R55 R56 R57 R58 R59 R60 R61 R62 R63 R64 R65 R66 R67 R68 R69 R70 R71 R72 R73 R74 R75 R76 R77 R78 R79 R80 R81 R82 R83 R84 R85 R86 R87 R88 R89 R90 R91 R92 R93 R94 R95 R96 R97 R98 R99 R100 R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R116 R117 R118 R119 R120 R121 R122 R123 R124 R125 R126 R127 R128 R129 R130 R131 R132 R133 R134 R135 R136 R137 R138 R139 R140 R141 R142 R143 R144 R145 R146 R147 R148 R149 R150 R151 R152 R153 R154 R155 R156 R157 R158 R159 R160 R161 R162 R163 R164 R165 R166 R167 R168 R169 R170 R171 R172 R173 R174 R175 R176 R177 R178 R179 R180 R181 R182 R183 R184 R185 R186 R187 R188 R189 R190 R191 R192 R193 R194 R195 R196 R197 R198 R199 R200 R201 R202 R203 R204 R205 R206 R207 R208 R209 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 S40 S41 S42 S43 S44 S45 S46 S47 S48 S49 S50 S51 S52 S53 S54 S55 S56 S57 S58 S59 S60 S61 S62 S63 S64 S65 S66 S67 S68 S69 S70 S71 S72 S73 S74 S75 S76 S77 S78 S79 S80 S81 S82 S83 S84 S85 S86 S87 S88 S89 S90 S91 S92 S93 S94 S95 S96 S97 S98 S99 S100 S101 S102 S103 S104 S105 S106 S107 S108 S109 S110 S111 S112 S113 S114 S115 S116 S117 S118 S119 S120 S121 S122 S123 S124 S125 S126 S127 S128 S129 S130 S131 S132 S133 S134 S135 S136 S137 S138 S139 S140 S141 S142 S143 S144 S145 S146 S147 S148 S149 S150 S151 S152 S153 S154 S155 S156 S157 S158 S159 S160 S161 S162 S163 S164 S165 S166 S167 S168 S169 S170 S171 S172 S173 S174 S175 S176 S177 S178 S179 S180 S181 S182 S183 S184 S185 S186 S187 S188 S189 S190 S191 S192 S193 S194 S195 S196 S197 S198 S199 S200 S201 S202 S203 S204 S205 S206 S207 S208 S209 T10 T11 T12 T13 T14 T15 T16 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T27 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 T41 T42 T43 T44 T45 T46 T47 T48 T49 T50 T51 T52 T53 T54 T55 T56 T57 T58 T59 T60 T61 T62 T63 T64 T65 T66 T67 T68 T69 T70 T71 T72 T73 T74 T75 T76 T77 T78 T79 T80 T81 T82 T83 T84 T85 T86 T87 T88 T89 T90 T91 T92 T93 T94 T95 T96 T97 T98 T99 T100 T101 T102 T103 T104 T105 T106 T107 T108 T109 T110 T111 T112 T113 T114 T115 T116 T117 T118 T119 T120 T121 T122 T123 T124 T125 T126 T127 T128 T129 T130 T131 T132 T133 T134 T135 T136 T137 T138 T139 T140 T141 T142 T143 T144 T145 T146 T147 T148 T149 T150 T151 T152 T153 T154 T155 T156 T157 T158 T159 T160 T161 T162 T163 T164 T165 T166 T167 T168 T169 T170 T171 T172 T173 T174 T175 T176 T177 T178 T179 T180 T181 T182 T183 T184 T185 T186 T187 T188 T189 T190 T191 T192 T193 T194 T195 T196 T197 T198 T199 T200 T201 T202 T203 T204 T205 T206 T207 T208 T209 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63 U64 U65 U66 U67 U68 U69 U70 U71 U72 U73 U74 U75 U76 U77 U78 U79 U80 U81 U82 U83 U84 U85 U86 U87 U88 U89 U90 U91 U92 U93 U94 U95 U96 U97 U98 U99 U100 U101 U102 U103 U104 U105 U106 U107 U108 U109 U110 U111 U112 U113 U114 U115 U116 U117 U118 U119 U120 U121 U122 U123 U124 U125 U126 U127 U128 U129 U130 U131 U132 U133 U134 U135 U136 U137 U138 U139 U140 U141 U142 U143 U144 U145 U146 U147 U148 U149 U150 U151 U152 U153 U154 U155 U156 U157 U158 U159 U160 U161 U162 U163 U164 U165 U166 U167 U168 U169 U170 U171 U172 U173 U174 U175 U176 U177 U178 U179 U180 U181 U182 U183 U184 U185 U186 U187 U188 U189 U190 U191 U192 U193 U194 U195 U196 U197 U198 U199 U200 U201 U202 U203 U204 U205 U206 U207 U208 U209 V10 V11 V12 V13 V14 V15 V16 V17 V18 V19 V20 V21 V22 V23 V24 V25 V26 V27 V28 V29 V30 V31 V32 V33 V34 V35 V36 V37 V38 V39 V40 V41 V42 V43 V44 V45 V46 V47 V48 V49 V50 V51 V52 V53 V54 V55 V56 V57 V58 V59 V60 V61 V62 V63 V64 V65 V66 V67 V68 V69 V70 V71 V72 V73 V74 V75 V76 V77 V78 V79 V80 V81 V82 V83 V84 V85 V86 V87 V88 V89 V90 V91 V92 V93 V94 V95 V96 V97 V98 V99 V100 V101 V102 V103 V104 V105 V106 V107 V108 V109 V110 V111 V112 V113 V114 V115 V116 V117 V118 V119 V120 V121 V122 V123 V124 V125 V126 V127 V128 V129 V130 V131 V132 V133 V134 V135 V136 V137 V138 V139 V140 V141 V142 V143 V144 V145 V146 V147 V148 V149 V150 V151 V152 V153 V154 V155 V156 V157 V158 V159 V160 V161 V162 V163 V164 V165 V166 V167 V168 V169 V170 V171 V172 V173 V174 V175 V176 V177 V178 V179 V180 V181 V182 V183 V184 V185 V186 V187 V188 V189 V190 V191 V192 V193 V194 V195 V196 V197 V198 V199 V200 V201 V202 V203 V204 V205 V206 V207 V208 V209 W10 W11 W12 W13 W14 W15 W16 W17 W18 W19 W20 W21 W22 W23 W24 W25 W26 W27 W28 W29 W30 W31 W32 W33 W34 W35 W36 W37 W38 W39 W40 W41 W42 W43 W44 W45 W46 W47 W48 W49 W50 W51 W52 W53 W54 W55 W56 W57 W58 W59 W60 W61 W62 W63 W64 W65 W66 W67 W68 W69 W70 W71 W72 W73 W74 W75 W76 W77 W78 W79 W80 W81 W82 W83 W84 W85 W86 W87 W88 W89 W90 W91 W92 W93 W94 W95 W96 W97 W98 W99 W100 W101 W102 W103 W104 W105 W106 W107 W108 W109 W110 W111 W112 W113 W114 W115 W116 W117 W118 W119 W120 W121 W122 W123 W124 W125 W126 W127 W128 W129 W130 W131 W132 W133 W134 W135 W136 W137 W138 W139 W140 W141 W142 W143 W144 W145 W146 W147 W148 W149 W150 W151 W152 W153 W154 W155 W156 W157 W158 W159 W160 W161 W162 W163 W164 W165 W166 W167 W168 W169 W170 W171 W172 W173 W174 W175 W176 W177 W178 W179 W180 W181 W182 W183 W184 W185 W186 W187 W188 W189 W190 W191 W192 W193 W194 W195 W196 W197 W198 W199 W200 W201 W202 W203 W204 W205 W206 W207 W208 W209 X10 X11 X12 X13 X14 X15 X16 X17 X18 X19 X20 X21 X22 X23 X24 X25 X26 X27 X28 X29 X30 X31 X32 X33 X34 X35 X36 X37 X38 X39 X40 X41 X42 X43 X44 X45 X46 X47 X48 X49 X50 X51 X52 X53 X54 X55 X56 X57 X58 X59 X60 X61 X62 X63 X64 X65 X66 X67 X68 X69 X70 X71 X72 X73 X74 X75 X76 X77 X78 X79 X80 X81 X82 X83 X84 X85 X86 X87 X88 X89 X90 X91 X92 X93 X94 X95 X96 X97 X98 X99 X100 X101 X102 X103 X104 X105 X106 X107 X108 X109 X110 X111 X112 X113 X114 X115 X116 X117 X118 X119 X120 X121 X122 X123 X124 X125 X126 X127 X128 X129 X130 X131 X132 X133 X134 X135 X136 X137 X138 X139 X140 X141 X142 X143 X144 X145 X146 X147 X148 X149 X150 X151 X152 X153 X154 X155 X156 X157 X158 X159 X160 X161 X162 X163 X164 X165 X166 X167 X168 X169 X170 X171 X172 X173 X174 X175 X176 X177 X178 X179 X180 X181 X182 X183 X184 X185 X186 X187 X188 X189 X190 X191 X192 X193 X194 X195 X196 X197 X198 X199 X200 X201 X202 X203 X204 X205 X206 X207 X208 X209 Y10 Y11 Y12 Y13 Y14 Y15 Y16 Y17 Y18 Y19 Y20 Y21 Y22 Y23 Y24 Y25 Y26 Y27 Y28 Y29 Y30 Y31 Y32 Y33 Y34 Y35 Y36 Y37 Y38 Y39 Y40 Y41 Y42 Y43 Y44 Y45 Y46 Y47 Y48 Y49 Y50 Y51 Y52 Y53 Y54 Y55 Y56 Y57 Y58 Y59 Y60 Y61 Y62 Y63 Y64 Y65 Y66 Y67 Y68 Y69 Y70 Y71 Y72 Y73 Y74 Y75 Y76 Y77 Y78 Y79 Y80 Y81 Y82 Y83 Y84 Y85 Y86 Y87 Y88 Y89 Y90 Y91 Y92 Y93 Y94 Y95 Y96 Y97 Y98 Y99 Y100 Y101 Y102 Y103 Y104 Y105 Y106 Y107 Y108 Y109 Y110 Y111 Y112 Y113 Y114 Y115 Y116 Y117 Y118 Y119 Y120 Y121 Y122 Y123 Y124 Y125 Y126 Y127 Y128 Y129 Y130 Y131 Y132 Y133 Y134 Y135 Y136 Y137 Y138 Y139 Y140 Y141 Y142 Y143 Y144 Y145 Y146 Y147 Y148 Y149 Y150 Y151 Y152 Y153 Y154 Y155 Y156 Y157 Y158 Y159 Y160 Y161 Y162 Y163 Y164 Y165 Y166 Y167 Y168 Y169 Y170 Y171 Y172 Y173 Y174 Y175 Y176 Y177 Y178 Y179 Y180 Y181 Y182 Y183 Y184 Y185 Y186 Y187 Y188 Y189 Y190 Y191 Y192 Y193 Y194 Y195 Y196 Y197 Y198 Y199 Y200 Y201 Y202 Y203 Y204 Y205 Y206 Y207 Y208 Y209 Z10 Z11 Z12 Z13 Z14 Z15 Z16 Z17 Z18 Z19 Z20 Z21 Z22 Z23 Z24 Z25 Z26 Z27 Z28 Z29 Z30 Z31 Z32 Z33 Z34 Z35 Z36 Z37 Z38 Z39 Z40 Z41 Z42 Z43 Z44 Z45 Z46 Z47 Z48 Z49 Z50 Z51 Z52 Z53 Z54 Z55 Z56 Z57 Z58 Z59 Z60 Z61 Z62 Z63 Z64 Z65 Z66 Z67 Z68 Z69 Z70 Z71 Z72 Z73 Z74 Z75 Z76 Z77 Z78 Z79 Z80 Z81 Z82 Z83 Z84 Z85 Z86 Z87 Z88 Z89 Z90 Z91 Z92 Z93 Z94 Z95 Z96 Z97 Z98 Z99 Z100 Z101 Z102 Z103 Z104 Z105 Z106 Z107 Z108 Z109 Z110 Z111 Z112 Z113 Z114 Z115 Z116 Z117 Z118 Z119 Z120 Z121 Z122 Z123 Z124 Z125 Z126 Z127 Z128 Z129 Z130 Z131 Z132 Z133 Z134 Z135 Z136 Z137 Z138 Z139 Z140 Z141 Z142 Z143 Z144 Z145 Z146 Z147 Z148 Z149 Z150 Z151 Z152 Z153 Z154 Z155 Z156 Z157 Z158 Z159 Z160 Z161 Z162 Z163 Z164 Z165 Z166 Z167 Z168 Z169 Z170 Z171 Z172 Z173 Z174 Z175 Z176 Z177 Z178 Z179 Z180 Z181 Z182 Z183 Z184 Z185 Z186 Z187 Z188 Z189 Z190 Z191 Z192 Z193 Z194 Z195 Z196 Z197 Z198 Z199 Z200 Z201 Z202 Z203 Z204 Z205 Z206 Z207 Z208 Z209 AA10 AA11 AA12 AA13 AA14 AA15 AA16 AA17 AA18 AA19 AA20 AA21 AA22 AA23 AA24 AA25 AA26 AA27 AA28 AA29 AA30 AA31 AA32 AA33 AA34 AA35 AA36 AA37 AA38 AA39 AA40 AA41 AA42 AA43 AA44 AA45 AA46 AA47 AA48 AA49 AA50 AA51 AA52 AA53 AA54 AA55 AA56 AA57 AA58 AA59 AA60 AA61 AA62 AA63 AA64 AA65 AA66 AA67 AA68 AA69 AA70 AA71 AA72 AA73 AA74 AA75 AA76 AA77 AA78 AA79 AA80 AA81 AA82 AA83 AA84 AA85 AA86 AA87 AA88 AA89 AA90 AA91 AA92 AA93 AA94 AA95 AA96 AA97 AA98 AA99 AA100 AA101 AA102 AA103 AA104 AA105 AA106 AA107 AA108 AA109 AA110 AA111 AA112 AA113 AA114 AA115 AA116 AA117 AA118 AA119 AA120 AA121 AA122 AA123 AA124 AA125 AA126 AA127 AA128 AA129 AA130 AA131 AA132 AA133 AA134 AA135 AA136 AA137 AA138 AA139 AA140 AA141 AA142 AA143 AA144 AA145 AA146 AA147 AA148 AA149 AA150 AA151 AA152 AA153 AA154 AA155 AA156 AA157 AA158 AA159 AA160 AA161 AA162 AA163 AA164 AA165 AA166 AA167 AA168 AA169 AA170 AA171 AA172 AA173 AA174 AA175 AA176 AA177 AA178 AA179 AA180 AA181 AA182 AA183 AA184 AA185 AA186 AA187 AA188 AA189 AA190 AA191 AA192 AA193 AA194 AA195 AA196 AA197 AA198 AA199 AA200 AA201 AA202 AA203 AA204 AA205 AA206 AA207 AA208 AA209 AB10 AB11 AB12 AB13 AB14 AB15 AB16 AB17 AB18 AB19 AB20 AB21 AB22 AB23 AB24 AB25 AB26 AB27 AB28 AB29 AB30 AB31 AB32 AB33 AB34 AB35 AB36 AB37 AB38 AB39 AB40 AB41 AB42 AB43 AB44 AB45 AB46 AB47 AB48 AB49 AB50 AB51 AB52 AB53 AB54 AB55 AB56 AB57 AB58 AB59 AB60 AB61 AB62 AB63 AB64 AB65 AB66 AB67 AB68 AB69 AB70 AB71 AB72 AB73 AB74 AB75 AB76 AB77 AB78 AB79 AB80 AB81 AB82 AB83 AB84 AB85 AB86 AB87 AB88 AB89 AB90 AB91 AB92 AB93 AB94 AB95 AB96 AB97 AB98 AB99 AB100 AB101 AB102 AB103 AB104 AB105 AB106 AB107 AB108 AB109 AB110 AB111 AB112 AB113 AB114 AB115 AB116 AB117 AB118 AB119 AB120 AB121 AB122 AB123 AB124 AB125 AB126 AB127 AB128 AB129 AB130 AB131 AB132 AB133 AB134 AB135 AB136 AB137 AB138 AB139 AB140 AB141 AB142 AB143 AB144 AB145 AB146 AB147 AB148 AB149 AB150 AB151 AB152 AB153 AB154 AB155 AB156 AB157 AB158 AB159 AB160 AB161 AB162 AB163 AB164 AB165 AB166 AB167 AB168 AB169 AB170 AB171 AB172 AB173 AB174 AB175 AB176 AB177 AB178 AB179 AB180 AB181 AB182 AB183 AB184 AB185 AB186 AB187 AB188 AB189 AB190 AB191 AB192 AB193 AB194 AB195 AB196 AB197 AB198 AB199 AB200 AB201 AB202 AB203 AB204 AB205 AB206 AB207 AB208 AB209 AC10 AC11 AC12 AC13 AC14 AC15 AC16 AC17 AC18 AC19 AC20 AC21 AC22 AC23 AC24 AC25 AC26 AC27 AC28 AC29 AC30 AC31 AC32 AC33 AC34 AC35 AC36 AC37 AC38 AC39 AC40 AC41 AC42 AC43 AC44 AC45 AC46 AC47 AC48 AC49 AC50 AC51 AC52 AC53 AC54 AC55 AC56 AC57 AC58 AC59 AC60 AC61 AC62 AC63 AC64 AC65 AC66 AC67 AC68 AC69 AC70 AC71 AC72 AC73 AC74 AC75 AC76 AC77 AC78 AC79 AC80 AC81 AC82 AC83 AC84 AC85 AC86 AC87 AC88 AC89 AC90 AC91 AC92 AC93 AC94 AC95 AC96 AC97 AC98 AC99 AC100 AC101 AC102 AC103 AC104 AC105 AC106 AC107 AC108 AC109 AC110 AC111 AC112 AC113 AC114 AC115 AC116 AC117 AC118 AC119 AC120 AC121 AC122 AC123 AC124 AC125 AC126 AC127 AC128 AC129 AC130 AC131 AC132 AC133 AC134 AC135 AC136 AC137 AC138 AC139 AC140 AC141 AC142 AC143 AC144 AC145 AC146 AC147 AC148 AC149 AC150 AC151 AC152 AC153 AC154 AC155 AC156 AC157 AC158 AC159 AC160 AC161 AC162 AC163 AC164 AC165 AC166 AC167 AC168 AC169 AC170 AC171 AC172 AC173 AC174 AC175 AC176 AC177 AC178 AC179 AC180 AC181 AC182 AC183 AC184 AC185 AC186 AC187 AC188 AC189 AC190 AC191 AC192 AC193 AC194 AC195 AC196 AC197 AC198 AC199 AC200 AC201 AC202 AC203 AC204 AC205 AC206 AC207 AC208 AC209 AD10 AD11 AD12 AD13 AD14 AD15 AD16 AD17 AD18 AD19 AD20 AD21 AD22 AD23 AD24 AD25 AD26 AD27 AD28 AD29 AD30 AD31 AD32 AD33 AD34 AD35 AD36 AD37 AD38 AD39 AD40 AD41 AD42 AD43 AD44 AD45 AD46 AD47 AD48 AD49 AD50 AD51 AD52 AD53 AD54 AD55 AD56 AD57 AD58 AD59 AD60 AD61 AD62 AD63 AD64 AD65 AD66 AD67 AD68 AD69 AD70 AD71 AD72 AD73 AD74 AD75 AD76 AD77 AD78 AD79 AD80 AD81 AD82 AD83 AD84 AD85 AD86 AD87 AD88 AD89 AD90 AD91 AD92 AD93 AD94 AD95 AD96 AD97 AD98 AD99 AD100 AD101 AD102 AD103 AD104 AD105 AD106 AD107 AD108 AD109 AD110 AD111 AD112 AD113 AD114 AD115 AD116 AD117 AD118 AD119 AD120 AD121 AD122 AD123 AD124 AD125 AD126 AD127 AD128 AD129 AD130 AD131 AD132 AD133 AD134 AD135 AD136 AD137 AD138 AD139 AD140 AD141 AD142 AD143 AD144 AD145 AD146 AD147 AD148 AD149 AD150 AD151 AD152 AD153 AD154 AD155 AD156 AD157 AD158 AD159 AD160 AD161 AD162 AD163 AD164 AD165 AD166 AD167 AD168 AD169 AD170 AD171 AD172 AD173 AD174 AD175 AD176 AD177 AD178 AD179 AD180 AD181 AD182 AD183 AD184 AD185 AD186 AD187 AD188 AD189 AD190 AD191 AD192 AD193 AD194 AD195 AD196 AD197 AD198 AD199 AD200 AD201 AD202 AD203 AD204 AD205 AD206 AD207 AD208 AD209 AE10 AE11 AE12 AE13 AE14 AE15 AE16 AE17 AE18 AE19 AE20 AE21 AE22 AE23 AE24 AE25 AE26 AE27 AE28 AE29 AE30 AE31 AE32 AE33 AE34 AE35 AE36 AE37 AE38 AE39 AE40 AE41 AE42 AE43 AE44 AE45 AE46 AE47 AE48 AE49 AE50 AE51 AE52 AE53 AE54 AE55 AE56 AE57 AE58 AE59 AE60 AE61 AE62 AE63 AE64 AE65 AE66 AE67 AE68 AE69 AE70 AE71 AE72 AE73 AE74 AE75 AE76 AE77 AE78 AE79 AE80 AE81 AE82 AE83 AE84 AE85 AE86 AE87 AE88 AE89 AE90 AE91 AE92 AE93 AE94 AE95 AE96 AE97 AE98 AE99 AE100 AE101 AE102 AE103 AE104 AE105 AE106 AE107 AE108 AE109 AE110 AE111 AE112 AE113 AE114 AE115 AE116 AE117 AE118 AE119 AE120 AE121 AE122 AE123 AE124 AE125 AE126 AE127 AE128 AE129 AE130 AE131 AE132 AE133 AE134 AE135 AE136 AE137 AE138 AE139 AE140 AE141 AE142 AE143 AE144 AE145 AE146 AE147 AE148 AE149 AE150 AE151 AE152 AE153 AE154 AE155 AE156 AE157 AE158 AE159 AE160 AE161 AE162 AE163 AE164 AE165 AE166 AE167 AE168 AE169 AE170 AE171 AE172 AE173 AE174 AE175 AE176 AE177 AE178 AE179 AE180 AE181 AE182 AE183 AE184 AE185 AE186 AE187 AE188 AE189 AE190 AE191 AE192 AE193 AE194 AE195 AE196 AE197 AE198 AE199 AE200 AE201 AE202 AE203 AE204 AE205 AE206 AE207 AE208 AE209 AF10 AF11 AF12 AF13 AF14 AF15 AF16 AF17 AF18 AF19 AF20 AF21 AF22 AF23 AF24 AF25 AF26 AF27 AF28 AF29 AF30 AF31 AF32 AF33 AF34 AF35 AF36 AF37 AF38 AF39 AF40 AF41 AF42 AF43 AF44 AF45 AF46 AF47 AF48 AF49 AF50 AF51 AF52 AF53 AF54 AF55 AF56 AF57 AF58 AF59 AF60 AF61 AF62 AF63 AF64 AF65 AF66 AF67 AF68 AF69 AF70 AF71 AF72 AF73 AF74 AF75 AF76 AF77 AF78 AF79 AF80 AF81 AF82 AF83 AF84 AF85 AF86 AF87 AF88 AF89 AF90 AF91 AF92 AF93 AF94 AF95 AF96 AF97 AF98 AF99 AF100 AF101 AF102 AF103 AF104 AF105 AF106 AF107 AF108 AF109 AF110 AF111 AF112 AF113 AF114 AF115 AF116 AF117 AF118 AF119 AF120 AF121 AF122 AF123 AF124 AF125 AF126 AF127 AF128 AF129 AF130 AF131 AF132 AF133 AF134 AF135 AF136 AF137 AF138 AF139 AF140 AF141 AF142 AF143 AF144 AF145 AF146 AF147 AF148 AF149 AF150 AF151 AF152 AF153 AF154 AF155 AF156 AF157 AF158 AF159 AF160 AF161 AF162 AF163 AF164 AF165 AF166 AF167 AF168 AF169 AF170 AF171 AF172 AF173 AF174 AF175 AF176 AF177 AF178 AF179 AF180 AF181 AF182 AF183 AF184 AF185 AF186 AF187 AF188 AF189 AF190 AF191 AF192 AF193 AF194 AF195 AF196 AF197 AF198 AF199 AF200 AF201 AF202 AF203 AF204 AF205 AF206 AF207 AF208 AF209 AG10 AG11 AG12 AG13 AG14 AG15 AG16 AG17 AG18 AG19 AG20 AG21 AG22 AG23 AG24 AG25 AG26 AG27 AG28 AG29 AG30 AG31 AG32 AG33 AG34 AG35 AG36 AG37 AG38 AG39 AG40 AG41 AG42 AG43 AG44 AG45 AG46 AG47 AG48 AG49 AG50 AG51 AG52 AG53 AG54 AG55 AG56 AG57 AG58 AG59 AG60 AG61 AG62 AG63 AG64 AG65 AG66 AG67 AG68 AG69 AG70 AG71 AG72 AG73 AG74 AG75 AG76 AG77 AG78 AG79 AG80 AG81 AG82 AG83 AG84 AG85 AG86 AG87 AG88 AG89 AG90 AG91 AG92 AG93 AG94 AG95 AG96 AG97 AG98 AG99 AG100 AG101 AG102 AG103 AG104 AG105 AG106 AG107 AG108 AG109 AG110 AG111 AG112 AG113 AG114 AG115 AG116 AG117 AG118 AG119 AG120 AG121 AG122 AG123 AG124 AG125 AG126 AG127 AG128 AG129 AG130 AG131 AG132 AG133 AG134 AG135 AG136 AG137 AG138 AG139 AG140 AG141 AG142 AG143 AG144 AG145 AG146 AG147 AG148 AG149 AG150 AG151 AG152 AG153 AG154 AG155 AG156 AG157 AG158 AG159 AG160 AG161 AG162 AG163 AG164 AG165 AG166 AG167 AG168 AG169 AG170 AG171 AG172 AG173 AG174 AG175 AG176 AG177 AG178 AG179 AG180 AG181 AG182 AG183 AG184 AG185 AG186 AG187 AG188 AG189 AG190 AG191 AG192 AG193 AG194 AG195 AG196 AG197 AG198 AG199 AG200 AG201 AG202 AG203 AG204 AG205 AG206 AG207 AG208 AG209 AH10 AH11 AH12 AH13 AH14 AH15 AH16 AH17 AH18 AH19 AH20 AH21 AH22 AH23 AH24 AH25 AH26 AH27 AH28 AH29 AH30 AH31 AH32 AH33 AH34 AH35 AH36 AH37 AH38 AH39 AH40 AH41 AH42 AH43 AH44 AH45 AH46 AH47 AH48 AH49 AH50 AH51 AH52 AH53 AH54 AH55 AH56 AH57 AH58 AH59 AH60 AH61 AH62 AH63 AH64 AH65 AH66 AH67 AH68 AH69 AH70 AH71 AH72 AH73 AH74 AH75 AH76 AH77 AH78 AH79 AH80 AH81 AH82 AH83 AH84 AH85 AH86 AH87 AH88 AH89 AH90 AH91 AH92 AH93 AH94 AH95 AH96 AH97 AH98 AH99 AH100 AH101 AH102 AH103 AH104 AH105 AH106 AH107 AH108 AH109 AH110 AH111 AH112 AH113 AH114 AH115 AH116 AH117 AH118 AH119 AH120 AH121 AH122 AH123 AH124 AH125 AH126 AH127 AH128 AH129 AH130 AH131 AH132 AH133 AH134 AH135 AH136 AH137 AH138 AH139 AH140 AH141 AH142 AH143 AH144 AH145 AH146 AH147 AH148 AH149 AH150 AH151 AH152 AH153 AH154 AH155 AH156 AH157 AH158 AH159 AH160 AH161 AH162 AH163 AH164 AH165 AH166 AH167 AH168 AH169 AH170 AH171 AH172 AH173 AH174 AH175 AH176 AH177 AH178 AH179 AH180 AH181 AH182 AH183 AH184 AH185 AH186 AH187 AH188 AH189 AH190 AH191 AH192 AH193 AH194 AH195 AH196 AH197 AH198 AH199 AH200 AH201 AH202 AH203 AH204 AH205 AH206 AH207 AH208 AH209 AI10 AI11 AI12 AI13 AI14 AI15 AI16 AI17 AI18 AI19 AI20 AI21 AI22 AI23 AI24 AI25 AI26 AI27 AI28 AI29 AI30 AI31 AI32 AI33 AI34 AI35 AI36 AI37 AI38 AI39 AI40 AI41 AI42 AI43 AI44 AI45 AI46 AI47 AI48 AI49 AI50 AI51 AI52 AI53 AI54 AI55 AI56 AI57 AI58 AI59 AI60 AI61 AI62 AI63 AI64 AI65 AI66 AI67 AI68 AI69 AI70 AI71 AI72 AI73 AI74 AI75 AI76 AI77 AI78 AI79 AI80 AI81 AI82 AI83 AI84 AI85 AI86 AI87 AI88 AI89 AI90 AI91 AI92 AI93 AI94 AI95 AI96 AI97 AI98 AI99 AI100 AI101 AI102 AI103 AI104 AI105 AI106 AI107 AI108 AI109 AI110 AI111 AI112 AI113 AI114 AI115 AI116 AI117 AI118 AI119 AI120 AI121 AI122 AI123 AI124 AI125 AI126 AI127 AI128 AI129 AI130 AI131 AI132 AI133 AI134 AI135 AI136 AI137 AI138 AI139 AI140 AI141 AI142 AI143 AI144 AI145 AI146 AI147 AI148 AI149 AI150 AI151 AI152 AI153 AI154 AI155 AI156 AI157 AI158 AI159 AI160 AI161 AI162 AI163 AI164 AI165 AI166 AI167 AI168 AI169 AI170 AI171 AI172 AI173 AI174 AI175 AI176 AI177 AI178 AI179 AI180 AI181 AI182 AI183 AI184 AI185 AI186 AI187 AI188 AI189 AI190 AI191 AI192 AI193 AI194 AI195 AI196 AI197 AI198 AI199 AI200 AI201 AI202 AI203 AI204 AI205 AI206 AI207 AI208 AI209 AJ10 AJ11 AJ12 AJ13 AJ14 AJ15 AJ16 AJ17 AJ18 AJ19 AJ20 AJ21 AJ22 AJ23 AJ24 AJ25 AJ26 AJ27 AJ28 AJ29 AJ30 AJ31 AJ32 AJ33 AJ34 AJ35 AJ36 AJ37 AJ38 AJ39 AJ40 AJ41 AJ42 AJ43 AJ44 AJ45 AJ46 AJ47 AJ48 AJ49 AJ50 AJ51 AJ52 AJ53 AJ54 AJ55 AJ56 AJ57 AJ58 AJ59 AJ60 AJ61 AJ62 AJ63 AJ64 AJ65 AJ66 AJ67 AJ68 AJ69 AJ70 AJ71 AJ72 AJ73 AJ74 AJ75 AJ76 AJ77 AJ78 AJ79 AJ80 AJ81 AJ82 AJ83 AJ84 AJ85 AJ86 AJ87 AJ88 AJ89 AJ90 AJ91 AJ92 AJ93 AJ94 AJ95 AJ96 AJ97 AJ98 AJ99 AJ100 AJ101 AJ102 AJ103 AJ104 AJ105 AJ106 AJ107 AJ108 AJ109 AJ110 AJ111 AJ112 AJ113 AJ114 AJ115 AJ116 AJ117 AJ118 AJ119 AJ120 AJ121 AJ122 AJ123 AJ124 AJ125 AJ126 AJ127 AJ128 AJ129 AJ130 AJ131 AJ132 AJ133 AJ134 AJ135 AJ136 AJ137 AJ138 AJ139 AJ140 AJ141 AJ142 AJ143 AJ144 AJ145 AJ146 AJ147 AJ148 AJ149 AJ150 AJ151 AJ152 AJ153 AJ154 AJ155 AJ156 AJ157 AJ158 AJ159 AJ160 AJ161 AJ162 AJ163 AJ164 AJ165 AJ166 AJ167 AJ168 AJ169 AJ170 AJ171 AJ172 AJ173 AJ174 AJ175 AJ176 AJ177 AJ178 AJ179 AJ180 AJ181 AJ182 AJ183 AJ184 AJ185 AJ186 AJ187 AJ188 AJ189 AJ190 AJ191 AJ192 AJ193 AJ194 AJ195 AJ196 AJ197 AJ198 AJ199 AJ200 AJ201 AJ202 AJ203 AJ204 AJ205 AJ206 AJ207 AJ208 AJ209 AK10 AK11 AK12 AK13 AK14 AK15 AK16 AK17 AK18 AK19 AK20 AK21 AK22 AK23 AK24 AK25 AK26 AK27 AK28 AK29 AK30 AK31 AK32 AK33 AK34 AK35 AK36 AK37 AK38 AK39 AK40 AK41 AK42 AK43 AK44 AK45 AK46 AK47 AK48 AK49 AK50 AK51 AK52 AK53 AK54 AK55 AK56 AK57 AK58 AK59 AK60 AK61 AK62 AK63 AK64 AK65 AK66 AK67 AK68 AK69 AK70 AK71 AK72 AK73 AK74 AK75 AK76 AK77 AK78 AK79 AK80 AK81 AK82 AK83 AK84 AK85 AK86 AK87 AK88 AK89 AK90 AK91 AK92 AK93 AK94 AK95 AK96 AK97 AK98 AK99 AK100 AK101 AK102 AK103 AK104 AK105 AK106 AK107 AK108 AK109 AK110 AK111 AK112 AK113 AK114 AK115 AK116 AK117 AK118 AK119 AK120 AK121 AK122 AK123 AK124 AK125 AK126 AK127 AK128 AK129 AK130 AK131 AK132 AK133 AK134 AK135 AK136 AK137 AK138 AK139 AK140 AK141 AK142 AK143 AK144 AK145 AK146 AK147 AK148 AK149 AK150 AK151 AK152 AK153 AK154 AK155 AK156 AK157 AK158 AK159 AK160 AK161 AK162 AK163 AK164 AK165 AK166 AK167 AK168 AK169 AK170 AK171 AK172 AK173 AK174 AK175 AK176 AK177 AK178 AK179 AK180 AK181 AK182 AK183 AK184 AK185 AK186 AK187 AK188 AK189 AK190 AK191 AK192 AK193 AK194 AK195 AK196 AK197 AK198 AK199 AK200 AK201 AK202 AK203 AK204 AK205 AK206 AK207 AK208 AK209 AL10 AL11 AL12 AL13 AL14 AL15 AL16 AL17 AL18 AL19 AL20 AL21 AL22 AL23 AL24 AL25 AL26 AL27 AL28 AL29 AL30 AL31 AL32 AL33 AL34 AL35 AL36 AL37 AL38 AL39 AL40 AL41 AL42 AL43 AL44 AL45 AL46 AL47 AL48 AL49 AL50 AL51 AL52 AL53 AL54 AL55 AL56 AL57 AL58 AL59 AL60 AL61 AL62 AL63 AL64 AL65 AL66 AL67 AL68 AL69 AL70 AL71 AL72 AL73 AL74 AL75 AL76 AL77 AL78 AL79 AL80 AL81 AL82 AL83 AL84 AL85 AL86 AL87 AL88 AL89 AL90 AL91 AL92 AL93 AL94 AL95 AL96 AL97 AL98 AL99 AL100 AL101 AL102 AL103 AL104 AL105 AL106 AL107 AL108 AL109 AL110 AL111 AL112 AL113 AL114 AL115 AL116 AL117 AL118 AL119 AL120 AL121 AL122 AL123 AL124 AL125 AL126 AL127 AL128 AL129 AL130 AL131 AL132 AL133 AL134 AL135 AL136 AL137 AL138 AL139 AL140 AL141 AL142 AL143 AL144 AL145 AL146 AL147 AL148 AL149 AL150 AL151 AL152 AL153 AL154 AL155 AL156 AL157 AL158 AL159 AL160 AL161 AL162 AL163 AL164 AL165 AL166 AL167 AL168 AL169 AL170 AL171 AL172 AL173 AL174 AL175 AL176 AL177 AL178 AL179 AL180 AL181 AL182 AL183 AL184 AL185 AL186 AL187 AL188 AL189 AL190 AL191 AL192 AL193 AL194 AL195 AL196 AL197 AL198 AL199 AL200 AL201 AL202 AL203 AL204 AL205 AL206 AL207 AL208 AL209 AM10 AM11 AM12 AM13 AM14 AM15 AM16 AM17 AM18 AM19 AM20 AM21 AM22 AM23 AM24 AM25 AM26 AM27 AM28 AM29 AM30 AM31 AM32 AM33 AM34 AM35 AM36 AM37 AM38 AM39 AM40 AM41 AM42 AM43 AM44 AM45 AM46 AM47 AM48 AM49 AM50 AM51 AM52 AM53 AM54 AM55 AM56 AM57 AM58 AM59 AM60 AM61 AM62 AM63 AM64 AM65 AM66 AM67 AM68 AM69 AM70 AM71 AM72 AM73 AM74 AM75 AM76 AM77 AM78 AM79 AM80 AM81 AM82 AM83 AM84 AM85 AM86 AM87 AM88 AM89 AM90 AM91 AM92 AM93 AM94 AM95 AM96 AM97 AM98 AM99 AM100 AM101 AM102 AM103 AM104 AM105 AM106 AM107 AM108 AM109 AM110 AM111 AM112 AM113 AM114 AM115 AM116 AM117 AM118 AM119 AM120 AM121 AM122 AM123 AM124 AM125 AM126 AM127 AM128 AM129 AM130 AM131 AM132 AM133 AM134 AM135 AM136 AM137 AM138 AM139 AM140 AM141 AM142 AM143 AM144 AM145 AM146 AM147 AM148 AM149 AM150 AM151 AM152 AM153 AM154 AM155 AM156 AM157 AM158 AM159 AM160 AM161 AM162 AM163 AM164 AM165 AM166 AM167 AM168 AM169 AM170 AM171 AM172 AM173 AM174 AM175 AM176 AM177 AM178 AM179 AM180 AM181 AM182 AM183 AM184 AM185 AM186 AM187 AM188 AM189 AM190 AM191 AM192 AM193 AM194 AM195 AM196 AM197 AM198 AM199 AM200 AM201 AM202 AM203 AM204 AM205 AM206 AM207 AM208 AM209 AN10 AN11 AN12 AN13 AN14 AN15 AN16 AN17 AN18 AN19 AN20 AN21 AN22 AN23 AN24 AN25 AN26 AN27 AN28 AN29 AN30 AN31 AN32 AN33 AN34 AN35 AN36 AN37 AN38 AN39 AN40 AN41 AN42 AN43 AN44 AN45 AN46 AN47 AN48 AN49 AN50 AN51 AN52 AN53 AN54 AN55 AN56 AN57 AN58 AN59 AN60 AN61 AN62 AN63 AN64 AN65 AN66 AN67 AN68 AN69 AN70 AN71 AN72 AN73 AN74 AN75 AN76 AN77 AN78 AN79 AN80 AN81 AN82 AN83 AN84 AN85 AN86 AN87 AN88 AN89 AN90 AN91 AN92 AN93 AN94 AN95 AN96 AN97 AN98 AN99 AN100 AN101 AN102 AN103 AN104 AN105 AN106 AN107 AN108 AN109 AN110 AN111 AN112 AN113 AN114 AN115 AN116 AN117 AN118 AN119 AN120 AN121 AN122 AN123 AN124 AN125 AN126 AN127 AN128 AN129 AN130 AN131 AN132 AN133 AN134 AN135 AN136 AN137 AN138 AN139 AN140 AN141 AN142 AN143 AN144 AN145 AN146 AN147 AN148 AN149 AN150 AN151 AN152 AN153 AN154 AN155 AN156 AN157 AN158 AN159 AN160 AN161 AN162 AN163 AN164 AN165 AN166 AN167 AN168 AN169 AN170 AN171 AN172 AN173 AN174 AN175 AN176 AN177 AN178 AN179 AN180 AN181 AN182 AN183 AN184 AN185 AN186 AN187 AN188 AN189 AN190 AN191 AN192 AN193 AN194 AN195 AN196 AN197 AN198 AN199 AN200 AN201 AN202 AN203 AN204 AN205 AN206 AN207 AN208 AN209 AO10 AO11 AO12 AO13 AO14 AO15 AO16 AO17 AO18 AO19 AO20 AO21 AO22 AO23 AO24 AO25 AO26 AO27 AO28 AO29 AO30 AO31 AO32 AO33 AO34 AO35 AO36 AO37 AO38 AO39 AO40 AO41 AO42 AO43 AO44 AO45 AO46 AO47 AO48 AO49 AO50 AO51 AO52 AO53 AO54 AO55 AO56 AO57 AO58 AO59 AO60 AO61 AO62 AO63 AO64 AO65 AO66 AO67 AO68 AO69 AO70 AO71 AO72 AO73 AO74 AO75 AO76 AO77 AO78 AO79 AO80 AO81 AO82 AO83 AO84 AO85 AO86 AO87 AO88 AO89 AO90 AO91 AO92 AO93 AO94 AO95 AO96 AO97 AO98 AO99 AO100 AO101 AO102 AO103 AO104 AO105 AO106 AO107 AO108 AO109 AO110 AO111 AO112 AO113 AO114 AO115 AO116 AO117 AO118 AO119 AO120 AO121 AO122 AO123 AO124 AO125 AO126 AO127 AO128 AO129 AO130 AO131 AO132 AO133 AO134 AO135 AO136 AO137 AO138 AO139 AO140 AO141 AO142 AO143 AO144 AO145 AO146 AO147 AO148 AO149 AO150 AO151 AO152 AO153 AO154 AO155 AO156 AO157 AO158 AO159 AO160 AO161 AO162 AO163 AO164 AO165 AO166 AO167 AO168 AO169 AO170 AO171 AO172 AO173 AO174 AO175 AO176 AO177 AO178 AO179 AO180 AO181 AO182 AO183 AO184 AO185 AO186 AO187 AO188 AO189 AO190 AO191 AO192 AO193 AO194 AO195 AO196 AO197 AO198 AO199 AO200 AO201 AO202 AO203 AO204 AO205 AO206 AO207 AO208 AO209 AP10 AP11 AP12 AP13 AP14 AP15 AP16 AP17 AP18 AP19 AP20 AP21 AP22 AP23 AP24 AP25 AP26 AP27 AP28 AP29 AP30 AP31 AP32 AP33 AP34 AP35 AP36 AP37 AP38 AP39 AP40 AP41 AP42 AP43 AP44 AP45 AP46 AP47 AP48 AP49 AP50 AP51 AP52 AP53 AP54 AP55 AP56 AP57 AP58 AP59 AP60 AP61 AP62 AP63 AP64 AP65 AP66 AP67 AP68 AP69 AP70 AP71 AP72 AP73 AP74 AP75 AP76 AP77 AP78 AP79 AP80 AP81 AP82 AP83 AP84 AP85 AP86 AP87 AP88 AP89 AP90 AP91 AP92 AP93 AP94 AP95 AP96 AP97 AP98 AP99 AP100 AP101 AP102 AP103 AP104 AP105 AP106 AP107 AP108 AP109 AP110 AP111 AP112 AP113 AP114 AP115 AP116 AP117 AP118 AP119 AP120 AP121 AP122 AP123 AP124 AP125 AP126 AP127 AP128 AP129 AP130 AP131 AP132 AP133 AP134 AP135 AP136 AP137 AP138 AP139 AP140 AP141 AP142 AP143 AP144 AP145 AP146 AP147 AP148 AP149 AP150 AP151 AP152 AP153 AP154 AP155 AP156 AP157 AP158 AP159 AP160 AP161 AP162 AP163 AP164 AP165 AP166 AP167 AP168 AP169 AP170 AP171 AP172 AP173 AP174 AP175 AP176 AP177 AP178 AP179 AP180 AP181 AP182 AP183 AP184 AP185 AP186 AP187 AP188 AP189 AP190 AP191 AP192 AP193 AP194 AP195 AP196 AP197 AP198 AP199 AP200 AP201 AP202 AP203 AP204 AP205 AP206 AP207 AP208 AP209 AQ10 AQ11 AQ12 AQ13 AQ14 AQ15 AQ16 AQ17 AQ18 AQ19 AQ20 AQ21 AQ22 AQ23 AQ24 AQ25 AQ26 AQ27 AQ28 AQ29 AQ30 AQ31 AQ32 AQ33 AQ34 AQ35 AQ36 AQ37 AQ38 AQ39 AQ40 AQ41 AQ42 AQ43 AQ44 AQ45 AQ46 AQ47 AQ48 AQ49 AQ50 AQ51 AQ52 AQ53 AQ54 AQ55 AQ56 AQ57 AQ58 AQ59 AQ60 AQ61 AQ62 AQ63 AQ64 AQ65 AQ66 AQ67 AQ68 AQ69 AQ70 AQ71 AQ72 AQ73 AQ74 AQ75 AQ76 AQ77 AQ78 AQ79 AQ80 AQ81 AQ82 AQ83 AQ84 AQ85 AQ86 AQ87 AQ88 AQ89 AQ90 AQ91 AQ92 AQ93 AQ94 AQ95 AQ96 AQ97 AQ98 AQ99 AQ100 AQ101 AQ102 AQ103 AQ104 AQ105 AQ106 AQ107 AQ108 AQ109 AQ110 AQ111 AQ112 AQ113 AQ114 AQ115 AQ116 AQ117 AQ118 AQ119 AQ120 AQ121 AQ122 AQ123 AQ124 AQ125 AQ126 AQ127 AQ128 AQ129 AQ130 AQ131 AQ132 AQ133 AQ134 AQ135 AQ136 AQ137 AQ138 AQ139 AQ140 AQ141 AQ142 AQ143 AQ144 AQ145 AQ146 AQ147 AQ148 AQ149 AQ150 AQ151 AQ152 AQ153 AQ154 AQ155 AQ156 AQ157 AQ158 AQ159 AQ160 AQ161 AQ162 AQ163 AQ164 AQ165 AQ166 AQ167 AQ168 AQ169 AQ170 AQ171 AQ172 AQ173 AQ174 AQ175 AQ176 AQ177 AQ178 AQ179 AQ180 AQ181 AQ182 AQ183 AQ184 AQ185 AQ186 AQ187 AQ188 AQ189 AQ190 AQ191 AQ192 AQ193 AQ194 AQ195 AQ196 AQ197 AQ198 AQ199 AQ200 AQ201 AQ202 AQ203 AQ204 AQ205 AQ206 AQ207 AQ208 AQ209 AR10 AR11 AR12 AR13 AR14 AR15 AR16 AR17 AR18 AR19 AR20 AR21 AR22 AR23 AR24 AR25 AR26 AR27 AR28 AR29 AR30 AR31 AR32 AR33 AR34 AR35 AR36 AR37 AR38 AR39 AR40 AR41 AR42 AR43 AR44 AR45 AR46 AR47 AR48 AR49 AR50 AR51 AR52 AR53 AR54 AR55 AR56 AR57 AR58 AR59 AR60 AR61 AR62 AR63 AR64 AR65 AR66 AR67 AR68 AR69 AR70 AR71 AR72 AR73 AR74 AR75 AR76 AR77 AR78 AR79 AR80 AR81 AR82 AR83 AR84 AR85 AR86 AR87 AR88 AR89 AR90 AR91 AR92 AR93 AR94 AR95 AR96 AR97 AR98 AR99 AR100 AR101 AR102 AR103 AR104 AR105 AR106 AR107 AR108 AR109 AR110 AR111 AR112 AR113 AR114 AR115 AR116 AR117 AR118 AR119 AR120 AR121 AR122 AR123 AR124 AR125 AR126 AR127 AR128 AR129 AR130 AR131 AR132 AR133 AR134 AR135 AR136 AR137 AR138 AR139 AR140 AR141 AR142 AR143 AR144 AR145 AR146 AR147 AR148 AR149 AR150 AR151 AR152 AR153 AR154 AR155 AR156 AR157 AR158 AR159 AR160 AR161 AR162 AR163 AR164 AR165 AR166 AR167 AR168 AR169 AR170 AR171 AR172 AR173 AR174 AR175 AR176 AR177 AR178 AR179 AR180 AR181 AR182 AR183 AR184 AR185 AR186 AR187 AR188 AR189 AR190 AR191 AR192 AR193 AR194 AR195 AR196 AR197 AR198 AR199 AR200 AR201 AR202 AR203 AR204 AR205 AR206 AR207 AR208 AR209 AS10 AS11 AS12 AS13 AS14 AS15 AS16 AS17 AS18 AS19 AS20 AS21 AS22 AS23 AS24 AS25 AS26 AS27 AS28 AS29 AS30 AS31 AS32 AS33 AS34 AS35 AS36 AS37 AS38 AS39 AS40 AS41 AS42 AS43 AS44 AS45 AS46 AS47 AS48 AS49 AS50 AS51 AS52 AS53 AS54 AS55 AS56 AS57 AS58 AS59 AS60 AS61 AS62 AS63 AS64 AS65 AS66 AS67 AS68 AS69 AS70 AS71 AS72 AS73 AS74 AS75 AS76 AS77 AS78 AS79 AS80 AS81 AS82 AS83 AS84 AS85 AS86 AS87 AS88 AS89 AS90 AS91 AS92 AS93 AS94 AS95 AS96 AS97 AS98 AS99 AS100 AS101 AS102 AS103 AS104 AS105 AS106 AS107 AS108 AS109 AS110 AS111 AS112 AS113 AS114 AS115 AS116 AS117 AS118 AS119 AS120 AS121 AS122 AS123 AS124 AS125 AS126 AS127 AS128 AS129 AS130 AS131 AS132 AS133 AS134 AS135 AS136 AS137 AS138 AS139 AS140 AS141 AS142 AS143 AS144 AS145 AS146 AS147 AS148 AS149 AS150 AS151 AS152 AS153 AS154 AS155 AS156 AS157 AS158 AS159 AS160 AS161 AS162 AS163 AS164 AS165 AS166 AS167 AS168 AS169 AS170 AS171 AS172 AS173 AS174 AS175 AS176 AS177 AS178 AS179 AS180 AS181 AS182 AS183 AS184 AS185 AS186 AS187 AS188 AS189 AS190 AS191 AS192 AS193 AS194 AS195 AS196 AS197 AS198 AS199 AS200 AS201 AS202 AS203 AS204 AS205 AS206 AS207 AS208 AS209 AT10 AT11 AT12 AT13 AT14 AT15 AT16 AT17 AT18 AT19 AT20 AT21 AT22 AT23 AT24 AT25 AT26 AT27 AT28 AT29 AT30 AT31 AT32 AT33 AT34 AT35 AT36 AT37 AT38 AT39 AT40 AT41 AT42 AT43 AT44 AT45 AT46 AT47 AT48 AT49 AT50 AT51 AT52 AT53 AT54 AT55 AT56 AT57 AT58 AT59 AT60 AT61 AT62 AT63 AT64 AT65 AT66 AT67 AT68 AT69 AT70 AT71 AT72 AT73 AT74 AT75 AT76 AT77 AT78 AT79 AT80 AT81 AT82 AT83 AT84 AT85 AT86 AT87 AT88 AT89 AT90 AT91 AT92 AT93 AT94 AT95 AT96 AT97 AT98 AT99 AT100 AT101 AT102 AT103 AT104 AT105 AT106 AT107 AT108 AT109 AT110 AT111 AT112 AT113 AT114 AT115 AT116 AT117 AT118 AT119 AT120 AT121 AT122 AT123 AT124 AT125 AT126 AT127 AT128 AT129 AT130 AT131 AT132 AT133 AT134 AT135 AT136 AT137 AT138 AT139 AT140 AT141 AT142 AT143 AT144 AT145 AT146 AT147 AT148 AT149 AT150 AT151 AT152 AT153 AT154 AT155 AT156 AT157 AT158 AT159 AT160 AT161 AT162 AT163 AT164 AT165 AT166 AT167 AT168 AT169 AT170 AT171 AT172 AT173 AT174 AT175 AT176 AT177 AT178 AT179 AT180 AT181 AT182 AT183 AT184 AT185 AT186 AT187 AT188 AT189 AT190 AT191 AT192 AT193 AT194 AT195 AT196 AT197 AT198 AT199 AT200 AT201 AT202 AT203 AT204 AT205 AT206 AT207 AT208 AT209 AU10 AU11 AU12 AU13 AU14 AU15 AU16 AU17 AU18 AU19 AU20 AU21 AU22 AU23 AU24 AU25 AU26 AU27 AU28 AU29 AU30 AU31 AU32 AU33 AU34 AU35 AU36 AU37 AU38 AU39 AU40 AU41 AU42 AU43 AU44 AU45 AU46 AU47 AU48 AU49 AU50 AU51 AU52 AU53 AU54 AU55 AU56 AU57 AU58 AU59 AU60 AU61 AU62 AU63 AU64 AU65 AU66 AU67 AU68 AU69 AU70 AU71 AU72 AU73 AU74 AU75 AU76 AU77 AU78 AU79 AU80 AU81 AU82 AU83 AU84 AU85 AU86 AU87 AU88 AU89 AU90 AU91 AU92 AU93 AU94 AU95 AU96 AU97 AU98 AU99 AU100 AU101 AU102 AU103 AU104 AU105 AU106 AU107 AU108 AU109 AU110 AU111 AU112 AU113 AU114 AU115 AU116 AU117 AU118 AU119 AU120 AU121 AU122 AU123 AU124 AU125 AU126 AU127 AU128 AU129 AU130 AU131 AU132 AU133 AU134 AU135 AU136 AU137 AU138 AU139 AU140 AU141 AU142 AU143 AU144 AU145 AU146 AU147 AU148 AU149 AU150 AU151 AU152 AU153 AU154 AU155 AU156 AU157 AU158 AU159 AU160 AU161 AU162 AU163 AU164 AU165 AU166 AU167 AU168 AU169 AU170 AU171 AU172 AU173 AU174 AU175 AU176 AU177 AU178 AU179 AU180 AU181 AU182 AU183 AU184 AU185 AU186 AU187 AU188 AU189 AU190 AU191 AU192 AU193 AU194 AU195 AU196 AU197 AU198 AU199 AU200 AU201 AU202 AU203 AU204 AU205 AU206 AU207 AU208 AU209 AV10 AV11 AV12 AV13 AV14 AV15 AV16 AV17 AV18 AV19 AV20 AV21 AV22 AV23 AV24 AV25 AV26 AV27 AV28 AV29 AV30 AV31 AV32 AV33 AV34 AV35 AV36 AV37 AV38 AV39 AV40 AV41 AV42 AV43 AV44 AV45 AV46 AV47 AV48 AV49 AV50 AV51 AV52 AV53 AV54 AV55 AV56 AV57 AV58 AV59 AV60 AV61 AV62 AV63 AV64 AV65 AV66 AV67 AV68 AV69 AV70 AV71 AV72 AV73 AV74 AV75 AV76 AV77 AV78 AV79 AV80 AV81 AV82 AV83 AV84 AV85 AV86 AV87 AV88 AV89 AV90 AV91 AV92 AV93 AV94 AV95 AV96 AV97 AV98 AV99 AV100 AV101 AV102 AV103 AV104 AV105 AV106 AV107 AV108 AV109 AV110 AV111 AV112 AV113 AV114 AV115 AV116 AV117 AV118 AV119 AV120 AV121 AV122 AV123 AV124 AV125 AV126 AV127 AV128 AV129 AV130 AV131 AV132 AV133 AV134 AV135 AV136 AV137 AV138 AV139 AV140 AV141 AV142 AV143 AV144 AV145 AV146 AV147 AV148 AV149 AV150 AV151 AV152 AV153 AV154 AV155 AV156 AV157 AV158 AV159 AV160 AV161 AV162 AV163 AV164 AV165 AV166 AV167 AV168 AV169 AV170 AV171 AV172 AV173 AV174 AV175 AV176 AV177 AV178 AV179 AV180 AV181 AV182 AV183 AV184 AV185 AV186 AV187 AV188 AV189 AV190 AV191 AV192 AV193 AV194 AV195 AV196 AV197 AV198 AV199 AV200 AV201 AV202 AV203 AV204 AV205 AV206 AV207 AV208 AV209 AW10 AW11 AW12 AW13 AW14 AW15 AW16 AW17 AW18 AW19 AW20 AW21 AW22 AW23 AW24 AW25 AW26 AW27 AW28 AW29 AW30 AW31 AW32 AW33 AW34 AW35 AW36 AW37 AW38 AW39 AW40 AW41 AW42 AW43 AW44 AW45 AW46 AW47 AW48 AW49 AW50 AW51 AW52 AW53 AW54 AW55 AW56 AW57 AW58 AW59 AW60 AW61 AW62 AW63 AW64 AW65 AW66 AW67 AW68 AW69 AW70 AW71 AW72 AW73 AW74 AW75 AW76 AW77 AW78 AW79 AW80 AW81 AW82 AW83 AW84 AW85 AW86 AW87 AW88 AW89 AW90 AW91 AW92 AW93 AW94 AW95 AW96 AW97 AW98 AW99 AW100 AW101 AW102 AW103 AW104 AW105 AW106 AW107 AW108 AW109 AW110 AW111 AW112 AW113 AW114 AW115 AW116 AW117 AW118 AW119 AW120 AW121 AW122 AW123 AW124 AW125 AW126 AW127 AW128 AW129 AW130 AW131 AW132 AW133 AW134 AW135 AW136 AW137 AW138 AW139 AW140 AW141 AW142 AW143 AW144 AW145 AW146 AW147 AW148 AW149 AW150 AW151 AW152 AW153 AW154 AW155 AW156 AW157 AW158 AW159 AW160 AW161 AW162 AW163 AW164 AW165 AW166 AW167 AW168 AW169 AW170 AW171 AW172 AW173 AW174 AW175 AW176 AW177 AW178 AW179 AW180 AW181 AW182 AW183 AW184 AW185 AW186 AW187 AW188 AW189 AW190 AW191 AW192 AW193 AW194 AW195 AW196 AW197 AW198 AW199 AW200 AW201 AW202 AW203 AW204 AW205 AW206 AW207 AW208 AW209 AX10 AX11 AX12 AX13 AX14 AX15 AX16 AX17 AX18 AX19 AX20 AX21 AX22 AX23 AX24 AX25 AX26 AX27 AX28 AX29 AX30 AX31 AX32 AX33 AX34 AX35 AX36 AX37 AX38 AX39 AX40 AX41 AX42 AX43 AX44 AX45 AX46 AX47 AX48 AX49 AX50 AX51 AX52 AX53 AX54 AX55 AX56 AX57 AX58 AX59 AX60 AX61 AX62 AX63 AX64 AX65 AX66 AX67 AX68 AX69 AX70 AX71 AX72 AX73 AX74 AX75 AX76 AX77 AX78 AX79 AX80 AX81 AX82 AX83 AX84 AX85 AX86 AX87 AX88 AX89 AX90 AX91 AX92 AX93 AX94 AX95 AX96 AX97 AX98 AX99 AX100 AX101 AX102 AX103 AX104 AX105 AX106 AX107 AX108 AX109 AX110 AX111 AX112 AX113 AX114 AX115 AX116 AX117 AX118 AX119 AX120 AX121 AX122 AX123 AX124 AX125 AX126 AX127 AX128 AX129 AX130 AX131 AX132 AX133 AX134 AX135 AX136 AX137 AX138 AX139 AX140 AX141 AX142 AX143 AX144 AX145 AX146 AX147 AX148 AX149 AX150 AX151 AX152 AX153 AX154 AX155 AX156 AX157 AX158 AX159 AX160 AX161 AX162 AX163 AX164 AX165 AX166 AX167 AX168 AX169 AX170 AX171 AX172 AX173 AX174 AX175 AX176 AX177 AX178 AX179 AX180 AX181 AX182 AX183 AX184 AX185 AX186 AX187 AX188 AX189 AX190 AX191 AX192 AX193 AX194 AX195 AX196 AX197 AX198 AX199 AX200 AX201 AX202 AX203 AX204 AX205 AX206 AX207 AX208 AX209 AY10 AY11 AY12 AY13 AY14 AY15 AY16 AY17 AY18 AY19 AY20 AY21 AY22 AY23 AY24 AY25 AY26 AY27 AY28 AY29 AY30 AY31 AY32 AY33 AY34 AY35 AY36 AY37 AY38 AY39 AY40 AY41 AY42 AY43 AY44 AY45 AY46 AY47 AY48 AY49 AY50 AY51 AY52 AY53 AY54 AY55 AY56 AY57 AY58 AY59 AY60 AY61 AY62 AY63 AY64 AY65 AY66 AY67 AY68 AY69 AY70 AY71 AY72 AY73 AY74 AY75 AY76 AY77 AY78 AY79 AY80 AY81 AY82 AY83 AY84 AY85 AY86 AY87 AY88 AY89 AY90 AY91 AY92 AY93 AY94 AY95 AY96 AY97 AY98 AY99 AY100 AY101 AY102 AY103 AY104 AY105 AY106 AY107 AY108 AY109 AY110 AY111 AY112 AY113 AY114 AY115 AY116 AY117 AY118 AY119 AY120 AY121 AY122 AY123 AY124 AY125 AY126 AY127 AY128 AY129 AY130 AY131 AY132 AY133 AY134 AY135 AY136 AY137 AY138 AY139 AY140 AY141 AY142 AY143 AY144 AY145 AY146 AY147 AY148 AY149 AY150 AY151 AY152 AY153 AY154 AY155 AY156 AY157 AY158 AY159 AY160 AY161 AY162 AY163 AY164 AY165 AY166 AY167 AY168 AY169 AY170 AY171 AY172 AY173 AY174 AY175 AY176 AY177 AY178 AY179 AY180 AY181 AY182 AY183 AY184 AY185 AY186 AY187 AY188 AY189 AY190 AY191 AY192 AY193 AY194 AY195 AY196 AY197 AY198 AY199 AY200 AY201 AY202 AY203 AY204 AY205 AY206 AY207 AY208 AY209 AZ10 AZ11 AZ12 AZ13 AZ14 AZ15 AZ16 AZ17 AZ18 AZ19 AZ20 AZ21 AZ22 AZ23 AZ24 AZ25 AZ26 AZ27 AZ28 AZ29 AZ30 AZ31 AZ32 AZ33 AZ34 AZ35 AZ36 AZ37 AZ38 AZ39 AZ40 AZ41 AZ42 AZ43 AZ44 AZ45 AZ46 AZ47 AZ48 AZ49 AZ50 AZ51 AZ52 AZ53 AZ54 AZ55 AZ56 AZ57 AZ58 AZ59 AZ60 AZ61 AZ62 AZ63 AZ64 AZ65 AZ66 AZ67 AZ68 AZ69 AZ70 AZ71 AZ72 AZ73 AZ74 AZ75 AZ76 AZ77 AZ78 AZ79 AZ80 AZ81 AZ82 AZ83 AZ84 AZ85 AZ86 AZ87 AZ88 AZ89 AZ90 AZ91 AZ92 AZ93 AZ94 AZ95 AZ96 AZ97 AZ98 AZ99 AZ100 AZ101 AZ102 AZ103 AZ104 AZ105 AZ106 AZ107 AZ108 AZ109 AZ110 AZ111 AZ112 AZ113 AZ114 AZ115 AZ116 AZ117 AZ118 AZ119 AZ120 AZ121 AZ122 AZ123 AZ124 AZ125 AZ126 AZ127 AZ128 AZ129 AZ130 AZ131 AZ132 AZ133 AZ134 AZ135 AZ136 AZ137 AZ138 AZ139 AZ140 AZ141 AZ142 AZ143 AZ144 AZ145 AZ146 AZ147 AZ148 AZ149 AZ150 AZ151 AZ152 AZ153 AZ154 AZ155 AZ156 AZ157 AZ158 AZ159 AZ160 AZ161 AZ162 AZ163 AZ164 AZ165 AZ166 AZ167 AZ168 AZ169 AZ170 AZ171 AZ172 AZ173 AZ174 AZ175 AZ176 AZ177 AZ178 AZ179 AZ180 AZ181 AZ182 AZ183 AZ184 AZ185 AZ186 AZ187 AZ188 AZ189 AZ190 AZ191 AZ192 AZ193 AZ194 AZ195 AZ196 AZ197 AZ198 AZ199 AZ200 AZ201 AZ202 AZ203 AZ204 AZ205 AZ206 AZ207 AZ208 AZ209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Y,N,E"</formula1>
+      <formula1>"1,0,X"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21389,6 +21595,14 @@
           <t>TRANSACTIONS — All Money In &amp; Out</t>
         </is>
       </c>
+      <c r="B1" s="53" t="n"/>
+      <c r="C1" s="53" t="n"/>
+      <c r="D1" s="53" t="n"/>
+      <c r="E1" s="53" t="n"/>
+      <c r="F1" s="53" t="n"/>
+      <c r="G1" s="53" t="n"/>
+      <c r="H1" s="53" t="n"/>
+      <c r="I1" s="54" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
@@ -32680,6 +32894,13 @@
           <t>PLAYER BALANCES — Individual Ledger</t>
         </is>
       </c>
+      <c r="B1" s="53" t="n"/>
+      <c r="C1" s="53" t="n"/>
+      <c r="D1" s="53" t="n"/>
+      <c r="E1" s="53" t="n"/>
+      <c r="F1" s="53" t="n"/>
+      <c r="G1" s="53" t="n"/>
+      <c r="H1" s="54" t="n"/>
     </row>
     <row r="2" ht="14" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
@@ -35509,6 +35730,7 @@
           <t>DASHBOARD — Auto-calculated Summary (Website reads this)</t>
         </is>
       </c>
+      <c r="B1" s="54" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="42" t="inlineStr">
@@ -35516,6 +35738,7 @@
           <t>TEAM OVERVIEW</t>
         </is>
       </c>
+      <c r="B3" s="54" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -35568,6 +35791,7 @@
           <t>FINANCES</t>
         </is>
       </c>
+      <c r="B9" s="54" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -35653,6 +35877,7 @@
           <t>EVENTS</t>
         </is>
       </c>
+      <c r="B18" s="54" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -35761,7 +35986,9 @@
           <t>KEY &amp; INSTRUCTIONS</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="54" t="n"/>
+    </row>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="45" t="inlineStr">
         <is>
@@ -35881,7 +36108,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="52" t="inlineStr">
         <is>
-          <t>Y = Attended</t>
+          <t>1 = Attended | 0 = Absent | X = Exempt</t>
         </is>
       </c>
       <c r="B15" s="48" t="inlineStr">
@@ -35905,7 +36132,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
         <is>
-          <t>E = Excused</t>
+          <t>X = Exempt — absent but excused/exempt from cost</t>
         </is>
       </c>
       <c r="B17" s="48" t="inlineStr">
@@ -36100,4 +36327,896 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E107"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="58" t="inlineStr">
+        <is>
+          <t>🔒  ACCESS CODES — TREASURER ONLY  🔒</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="59" t="inlineStr">
+        <is>
+          <t>⚠️  HIDE THIS SHEET BEFORE SHARING THE FILE WITH PLAYERS  ⚠️</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="60" t="inlineStr">
+        <is>
+          <t>To hide: right-click this sheet tab → 'Hide'.  To unhide: right-click any tab → 'Unhide'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>Player Name</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>Access Code</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr">
+        <is>
+          <t>Notes / Share Method</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Alex Johnson</t>
+        </is>
+      </c>
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>AJ2024</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>Texted 3/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Sam Rivera</t>
+        </is>
+      </c>
+      <c r="B7" s="62" t="inlineStr">
+        <is>
+          <t>SR2024</t>
+        </is>
+      </c>
+      <c r="C7" s="63" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="D7" s="63" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Emailed 3/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Jordan Lee</t>
+        </is>
+      </c>
+      <c r="B8" s="64" t="inlineStr">
+        <is>
+          <t>JL2024</t>
+        </is>
+      </c>
+      <c r="C8" s="65" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="D8" s="65" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>Texted 3/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="66" t="inlineStr">
+        <is>
+          <t>Coach Kim</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="inlineStr">
+        <is>
+          <t>CK2024</t>
+        </is>
+      </c>
+      <c r="C9" s="68" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="D9" s="68" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E9" s="66" t="inlineStr">
+        <is>
+          <t>Hand delivered</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Taylor Smith</t>
+        </is>
+      </c>
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>TS2024</t>
+        </is>
+      </c>
+      <c r="C10" s="63" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="D10" s="63" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>Texted 3/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="69" t="n"/>
+      <c r="B11" s="70" t="n"/>
+      <c r="C11" s="71" t="n"/>
+      <c r="D11" s="71" t="n"/>
+      <c r="E11" s="69" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="72" t="n"/>
+      <c r="B12" s="73" t="n"/>
+      <c r="C12" s="74" t="n"/>
+      <c r="D12" s="74" t="n"/>
+      <c r="E12" s="72" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="69" t="n"/>
+      <c r="B13" s="70" t="n"/>
+      <c r="C13" s="71" t="n"/>
+      <c r="D13" s="71" t="n"/>
+      <c r="E13" s="69" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="72" t="n"/>
+      <c r="B14" s="73" t="n"/>
+      <c r="C14" s="74" t="n"/>
+      <c r="D14" s="74" t="n"/>
+      <c r="E14" s="72" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="69" t="n"/>
+      <c r="B15" s="70" t="n"/>
+      <c r="C15" s="71" t="n"/>
+      <c r="D15" s="71" t="n"/>
+      <c r="E15" s="69" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="72" t="n"/>
+      <c r="B16" s="73" t="n"/>
+      <c r="C16" s="74" t="n"/>
+      <c r="D16" s="74" t="n"/>
+      <c r="E16" s="72" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="69" t="n"/>
+      <c r="B17" s="70" t="n"/>
+      <c r="C17" s="71" t="n"/>
+      <c r="D17" s="71" t="n"/>
+      <c r="E17" s="69" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="72" t="n"/>
+      <c r="B18" s="73" t="n"/>
+      <c r="C18" s="74" t="n"/>
+      <c r="D18" s="74" t="n"/>
+      <c r="E18" s="72" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="69" t="n"/>
+      <c r="B19" s="70" t="n"/>
+      <c r="C19" s="71" t="n"/>
+      <c r="D19" s="71" t="n"/>
+      <c r="E19" s="69" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="72" t="n"/>
+      <c r="B20" s="73" t="n"/>
+      <c r="C20" s="74" t="n"/>
+      <c r="D20" s="74" t="n"/>
+      <c r="E20" s="72" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="69" t="n"/>
+      <c r="B21" s="70" t="n"/>
+      <c r="C21" s="71" t="n"/>
+      <c r="D21" s="71" t="n"/>
+      <c r="E21" s="69" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="72" t="n"/>
+      <c r="B22" s="73" t="n"/>
+      <c r="C22" s="74" t="n"/>
+      <c r="D22" s="74" t="n"/>
+      <c r="E22" s="72" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="69" t="n"/>
+      <c r="B23" s="70" t="n"/>
+      <c r="C23" s="71" t="n"/>
+      <c r="D23" s="71" t="n"/>
+      <c r="E23" s="69" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="72" t="n"/>
+      <c r="B24" s="73" t="n"/>
+      <c r="C24" s="74" t="n"/>
+      <c r="D24" s="74" t="n"/>
+      <c r="E24" s="72" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="69" t="n"/>
+      <c r="B25" s="70" t="n"/>
+      <c r="C25" s="71" t="n"/>
+      <c r="D25" s="71" t="n"/>
+      <c r="E25" s="69" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="72" t="n"/>
+      <c r="B26" s="73" t="n"/>
+      <c r="C26" s="74" t="n"/>
+      <c r="D26" s="74" t="n"/>
+      <c r="E26" s="72" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="69" t="n"/>
+      <c r="B27" s="70" t="n"/>
+      <c r="C27" s="71" t="n"/>
+      <c r="D27" s="71" t="n"/>
+      <c r="E27" s="69" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="72" t="n"/>
+      <c r="B28" s="73" t="n"/>
+      <c r="C28" s="74" t="n"/>
+      <c r="D28" s="74" t="n"/>
+      <c r="E28" s="72" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="69" t="n"/>
+      <c r="B29" s="70" t="n"/>
+      <c r="C29" s="71" t="n"/>
+      <c r="D29" s="71" t="n"/>
+      <c r="E29" s="69" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="72" t="n"/>
+      <c r="B30" s="73" t="n"/>
+      <c r="C30" s="74" t="n"/>
+      <c r="D30" s="74" t="n"/>
+      <c r="E30" s="72" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="69" t="n"/>
+      <c r="B31" s="70" t="n"/>
+      <c r="C31" s="71" t="n"/>
+      <c r="D31" s="71" t="n"/>
+      <c r="E31" s="69" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="72" t="n"/>
+      <c r="B32" s="73" t="n"/>
+      <c r="C32" s="74" t="n"/>
+      <c r="D32" s="74" t="n"/>
+      <c r="E32" s="72" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="69" t="n"/>
+      <c r="B33" s="70" t="n"/>
+      <c r="C33" s="71" t="n"/>
+      <c r="D33" s="71" t="n"/>
+      <c r="E33" s="69" t="n"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="72" t="n"/>
+      <c r="B34" s="73" t="n"/>
+      <c r="C34" s="74" t="n"/>
+      <c r="D34" s="74" t="n"/>
+      <c r="E34" s="72" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="69" t="n"/>
+      <c r="B35" s="70" t="n"/>
+      <c r="C35" s="71" t="n"/>
+      <c r="D35" s="71" t="n"/>
+      <c r="E35" s="69" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="72" t="n"/>
+      <c r="B36" s="73" t="n"/>
+      <c r="C36" s="74" t="n"/>
+      <c r="D36" s="74" t="n"/>
+      <c r="E36" s="72" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="69" t="n"/>
+      <c r="B37" s="70" t="n"/>
+      <c r="C37" s="71" t="n"/>
+      <c r="D37" s="71" t="n"/>
+      <c r="E37" s="69" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="72" t="n"/>
+      <c r="B38" s="73" t="n"/>
+      <c r="C38" s="74" t="n"/>
+      <c r="D38" s="74" t="n"/>
+      <c r="E38" s="72" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="69" t="n"/>
+      <c r="B39" s="70" t="n"/>
+      <c r="C39" s="71" t="n"/>
+      <c r="D39" s="71" t="n"/>
+      <c r="E39" s="69" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="72" t="n"/>
+      <c r="B40" s="73" t="n"/>
+      <c r="C40" s="74" t="n"/>
+      <c r="D40" s="74" t="n"/>
+      <c r="E40" s="72" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="69" t="n"/>
+      <c r="B41" s="70" t="n"/>
+      <c r="C41" s="71" t="n"/>
+      <c r="D41" s="71" t="n"/>
+      <c r="E41" s="69" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="72" t="n"/>
+      <c r="B42" s="73" t="n"/>
+      <c r="C42" s="74" t="n"/>
+      <c r="D42" s="74" t="n"/>
+      <c r="E42" s="72" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="69" t="n"/>
+      <c r="B43" s="70" t="n"/>
+      <c r="C43" s="71" t="n"/>
+      <c r="D43" s="71" t="n"/>
+      <c r="E43" s="69" t="n"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="72" t="n"/>
+      <c r="B44" s="73" t="n"/>
+      <c r="C44" s="74" t="n"/>
+      <c r="D44" s="74" t="n"/>
+      <c r="E44" s="72" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="69" t="n"/>
+      <c r="B45" s="70" t="n"/>
+      <c r="C45" s="71" t="n"/>
+      <c r="D45" s="71" t="n"/>
+      <c r="E45" s="69" t="n"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="72" t="n"/>
+      <c r="B46" s="73" t="n"/>
+      <c r="C46" s="74" t="n"/>
+      <c r="D46" s="74" t="n"/>
+      <c r="E46" s="72" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="69" t="n"/>
+      <c r="B47" s="70" t="n"/>
+      <c r="C47" s="71" t="n"/>
+      <c r="D47" s="71" t="n"/>
+      <c r="E47" s="69" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="72" t="n"/>
+      <c r="B48" s="73" t="n"/>
+      <c r="C48" s="74" t="n"/>
+      <c r="D48" s="74" t="n"/>
+      <c r="E48" s="72" t="n"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="69" t="n"/>
+      <c r="B49" s="70" t="n"/>
+      <c r="C49" s="71" t="n"/>
+      <c r="D49" s="71" t="n"/>
+      <c r="E49" s="69" t="n"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="72" t="n"/>
+      <c r="B50" s="73" t="n"/>
+      <c r="C50" s="74" t="n"/>
+      <c r="D50" s="74" t="n"/>
+      <c r="E50" s="72" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="69" t="n"/>
+      <c r="B51" s="70" t="n"/>
+      <c r="C51" s="71" t="n"/>
+      <c r="D51" s="71" t="n"/>
+      <c r="E51" s="69" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="72" t="n"/>
+      <c r="B52" s="73" t="n"/>
+      <c r="C52" s="74" t="n"/>
+      <c r="D52" s="74" t="n"/>
+      <c r="E52" s="72" t="n"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="69" t="n"/>
+      <c r="B53" s="70" t="n"/>
+      <c r="C53" s="71" t="n"/>
+      <c r="D53" s="71" t="n"/>
+      <c r="E53" s="69" t="n"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="72" t="n"/>
+      <c r="B54" s="73" t="n"/>
+      <c r="C54" s="74" t="n"/>
+      <c r="D54" s="74" t="n"/>
+      <c r="E54" s="72" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="69" t="n"/>
+      <c r="B55" s="70" t="n"/>
+      <c r="C55" s="71" t="n"/>
+      <c r="D55" s="71" t="n"/>
+      <c r="E55" s="69" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="72" t="n"/>
+      <c r="B56" s="73" t="n"/>
+      <c r="C56" s="74" t="n"/>
+      <c r="D56" s="74" t="n"/>
+      <c r="E56" s="72" t="n"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="69" t="n"/>
+      <c r="B57" s="70" t="n"/>
+      <c r="C57" s="71" t="n"/>
+      <c r="D57" s="71" t="n"/>
+      <c r="E57" s="69" t="n"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="72" t="n"/>
+      <c r="B58" s="73" t="n"/>
+      <c r="C58" s="74" t="n"/>
+      <c r="D58" s="74" t="n"/>
+      <c r="E58" s="72" t="n"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="69" t="n"/>
+      <c r="B59" s="70" t="n"/>
+      <c r="C59" s="71" t="n"/>
+      <c r="D59" s="71" t="n"/>
+      <c r="E59" s="69" t="n"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="72" t="n"/>
+      <c r="B60" s="73" t="n"/>
+      <c r="C60" s="74" t="n"/>
+      <c r="D60" s="74" t="n"/>
+      <c r="E60" s="72" t="n"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="69" t="n"/>
+      <c r="B61" s="70" t="n"/>
+      <c r="C61" s="71" t="n"/>
+      <c r="D61" s="71" t="n"/>
+      <c r="E61" s="69" t="n"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="72" t="n"/>
+      <c r="B62" s="73" t="n"/>
+      <c r="C62" s="74" t="n"/>
+      <c r="D62" s="74" t="n"/>
+      <c r="E62" s="72" t="n"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="69" t="n"/>
+      <c r="B63" s="70" t="n"/>
+      <c r="C63" s="71" t="n"/>
+      <c r="D63" s="71" t="n"/>
+      <c r="E63" s="69" t="n"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="72" t="n"/>
+      <c r="B64" s="73" t="n"/>
+      <c r="C64" s="74" t="n"/>
+      <c r="D64" s="74" t="n"/>
+      <c r="E64" s="72" t="n"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="69" t="n"/>
+      <c r="B65" s="70" t="n"/>
+      <c r="C65" s="71" t="n"/>
+      <c r="D65" s="71" t="n"/>
+      <c r="E65" s="69" t="n"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="72" t="n"/>
+      <c r="B66" s="73" t="n"/>
+      <c r="C66" s="74" t="n"/>
+      <c r="D66" s="74" t="n"/>
+      <c r="E66" s="72" t="n"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="69" t="n"/>
+      <c r="B67" s="70" t="n"/>
+      <c r="C67" s="71" t="n"/>
+      <c r="D67" s="71" t="n"/>
+      <c r="E67" s="69" t="n"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="72" t="n"/>
+      <c r="B68" s="73" t="n"/>
+      <c r="C68" s="74" t="n"/>
+      <c r="D68" s="74" t="n"/>
+      <c r="E68" s="72" t="n"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="69" t="n"/>
+      <c r="B69" s="70" t="n"/>
+      <c r="C69" s="71" t="n"/>
+      <c r="D69" s="71" t="n"/>
+      <c r="E69" s="69" t="n"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="72" t="n"/>
+      <c r="B70" s="73" t="n"/>
+      <c r="C70" s="74" t="n"/>
+      <c r="D70" s="74" t="n"/>
+      <c r="E70" s="72" t="n"/>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="69" t="n"/>
+      <c r="B71" s="70" t="n"/>
+      <c r="C71" s="71" t="n"/>
+      <c r="D71" s="71" t="n"/>
+      <c r="E71" s="69" t="n"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="72" t="n"/>
+      <c r="B72" s="73" t="n"/>
+      <c r="C72" s="74" t="n"/>
+      <c r="D72" s="74" t="n"/>
+      <c r="E72" s="72" t="n"/>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="69" t="n"/>
+      <c r="B73" s="70" t="n"/>
+      <c r="C73" s="71" t="n"/>
+      <c r="D73" s="71" t="n"/>
+      <c r="E73" s="69" t="n"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="72" t="n"/>
+      <c r="B74" s="73" t="n"/>
+      <c r="C74" s="74" t="n"/>
+      <c r="D74" s="74" t="n"/>
+      <c r="E74" s="72" t="n"/>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="69" t="n"/>
+      <c r="B75" s="70" t="n"/>
+      <c r="C75" s="71" t="n"/>
+      <c r="D75" s="71" t="n"/>
+      <c r="E75" s="69" t="n"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="72" t="n"/>
+      <c r="B76" s="73" t="n"/>
+      <c r="C76" s="74" t="n"/>
+      <c r="D76" s="74" t="n"/>
+      <c r="E76" s="72" t="n"/>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="69" t="n"/>
+      <c r="B77" s="70" t="n"/>
+      <c r="C77" s="71" t="n"/>
+      <c r="D77" s="71" t="n"/>
+      <c r="E77" s="69" t="n"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="72" t="n"/>
+      <c r="B78" s="73" t="n"/>
+      <c r="C78" s="74" t="n"/>
+      <c r="D78" s="74" t="n"/>
+      <c r="E78" s="72" t="n"/>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="69" t="n"/>
+      <c r="B79" s="70" t="n"/>
+      <c r="C79" s="71" t="n"/>
+      <c r="D79" s="71" t="n"/>
+      <c r="E79" s="69" t="n"/>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="72" t="n"/>
+      <c r="B80" s="73" t="n"/>
+      <c r="C80" s="74" t="n"/>
+      <c r="D80" s="74" t="n"/>
+      <c r="E80" s="72" t="n"/>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="69" t="n"/>
+      <c r="B81" s="70" t="n"/>
+      <c r="C81" s="71" t="n"/>
+      <c r="D81" s="71" t="n"/>
+      <c r="E81" s="69" t="n"/>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="72" t="n"/>
+      <c r="B82" s="73" t="n"/>
+      <c r="C82" s="74" t="n"/>
+      <c r="D82" s="74" t="n"/>
+      <c r="E82" s="72" t="n"/>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="69" t="n"/>
+      <c r="B83" s="70" t="n"/>
+      <c r="C83" s="71" t="n"/>
+      <c r="D83" s="71" t="n"/>
+      <c r="E83" s="69" t="n"/>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="72" t="n"/>
+      <c r="B84" s="73" t="n"/>
+      <c r="C84" s="74" t="n"/>
+      <c r="D84" s="74" t="n"/>
+      <c r="E84" s="72" t="n"/>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="69" t="n"/>
+      <c r="B85" s="70" t="n"/>
+      <c r="C85" s="71" t="n"/>
+      <c r="D85" s="71" t="n"/>
+      <c r="E85" s="69" t="n"/>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="72" t="n"/>
+      <c r="B86" s="73" t="n"/>
+      <c r="C86" s="74" t="n"/>
+      <c r="D86" s="74" t="n"/>
+      <c r="E86" s="72" t="n"/>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="69" t="n"/>
+      <c r="B87" s="70" t="n"/>
+      <c r="C87" s="71" t="n"/>
+      <c r="D87" s="71" t="n"/>
+      <c r="E87" s="69" t="n"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="72" t="n"/>
+      <c r="B88" s="73" t="n"/>
+      <c r="C88" s="74" t="n"/>
+      <c r="D88" s="74" t="n"/>
+      <c r="E88" s="72" t="n"/>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="69" t="n"/>
+      <c r="B89" s="70" t="n"/>
+      <c r="C89" s="71" t="n"/>
+      <c r="D89" s="71" t="n"/>
+      <c r="E89" s="69" t="n"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="72" t="n"/>
+      <c r="B90" s="73" t="n"/>
+      <c r="C90" s="74" t="n"/>
+      <c r="D90" s="74" t="n"/>
+      <c r="E90" s="72" t="n"/>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="69" t="n"/>
+      <c r="B91" s="70" t="n"/>
+      <c r="C91" s="71" t="n"/>
+      <c r="D91" s="71" t="n"/>
+      <c r="E91" s="69" t="n"/>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="72" t="n"/>
+      <c r="B92" s="73" t="n"/>
+      <c r="C92" s="74" t="n"/>
+      <c r="D92" s="74" t="n"/>
+      <c r="E92" s="72" t="n"/>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="69" t="n"/>
+      <c r="B93" s="70" t="n"/>
+      <c r="C93" s="71" t="n"/>
+      <c r="D93" s="71" t="n"/>
+      <c r="E93" s="69" t="n"/>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="72" t="n"/>
+      <c r="B94" s="73" t="n"/>
+      <c r="C94" s="74" t="n"/>
+      <c r="D94" s="74" t="n"/>
+      <c r="E94" s="72" t="n"/>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="69" t="n"/>
+      <c r="B95" s="70" t="n"/>
+      <c r="C95" s="71" t="n"/>
+      <c r="D95" s="71" t="n"/>
+      <c r="E95" s="69" t="n"/>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="72" t="n"/>
+      <c r="B96" s="73" t="n"/>
+      <c r="C96" s="74" t="n"/>
+      <c r="D96" s="74" t="n"/>
+      <c r="E96" s="72" t="n"/>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="69" t="n"/>
+      <c r="B97" s="70" t="n"/>
+      <c r="C97" s="71" t="n"/>
+      <c r="D97" s="71" t="n"/>
+      <c r="E97" s="69" t="n"/>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="72" t="n"/>
+      <c r="B98" s="73" t="n"/>
+      <c r="C98" s="74" t="n"/>
+      <c r="D98" s="74" t="n"/>
+      <c r="E98" s="72" t="n"/>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="69" t="n"/>
+      <c r="B99" s="70" t="n"/>
+      <c r="C99" s="71" t="n"/>
+      <c r="D99" s="71" t="n"/>
+      <c r="E99" s="69" t="n"/>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="72" t="n"/>
+      <c r="B100" s="73" t="n"/>
+      <c r="C100" s="74" t="n"/>
+      <c r="D100" s="74" t="n"/>
+      <c r="E100" s="72" t="n"/>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="69" t="n"/>
+      <c r="B101" s="70" t="n"/>
+      <c r="C101" s="71" t="n"/>
+      <c r="D101" s="71" t="n"/>
+      <c r="E101" s="69" t="n"/>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="72" t="n"/>
+      <c r="B102" s="73" t="n"/>
+      <c r="C102" s="74" t="n"/>
+      <c r="D102" s="74" t="n"/>
+      <c r="E102" s="72" t="n"/>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="69" t="n"/>
+      <c r="B103" s="70" t="n"/>
+      <c r="C103" s="71" t="n"/>
+      <c r="D103" s="71" t="n"/>
+      <c r="E103" s="69" t="n"/>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="72" t="n"/>
+      <c r="B104" s="73" t="n"/>
+      <c r="C104" s="74" t="n"/>
+      <c r="D104" s="74" t="n"/>
+      <c r="E104" s="72" t="n"/>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="69" t="n"/>
+      <c r="B105" s="70" t="n"/>
+      <c r="C105" s="71" t="n"/>
+      <c r="D105" s="71" t="n"/>
+      <c r="E105" s="69" t="n"/>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="75" t="inlineStr">
+        <is>
+          <t>💡 Tip: Codes can be anything — e.g. initials + jersey # + year.  Make them easy to remember but hard to guess.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A107:E107"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Active,Inactive,Alumni"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C86 C87 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C102 C103 C104 C105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Player,Captain,Coach,Treasurer,Manager"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>